<commit_message>
Ingest approved entries (2026-07-14)
</commit_message>
<xml_diff>
--- a/data/Trump_Second_Term_Weekly_Tracker.xlsx
+++ b/data/Trump_Second_Term_Weekly_Tracker.xlsx
@@ -6696,7 +6696,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="4" t="s">
         <v>516</v>
       </c>
@@ -6710,7 +6710,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="4" t="s">
         <v>516</v>
       </c>
@@ -6724,7 +6724,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="4" t="s">
         <v>516</v>
       </c>
@@ -6738,7 +6738,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="4" t="s">
         <v>516</v>
       </c>
@@ -6752,7 +6752,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="4" t="s">
         <v>516</v>
       </c>
@@ -6766,7 +6766,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="4" t="s">
         <v>516</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="4" t="s">
         <v>516</v>
       </c>
@@ -9342,7 +9342,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="5" t="n">
         <v>157</v>
       </c>
@@ -9359,7 +9359,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="5" t="n">
         <v>158</v>
       </c>
@@ -9376,7 +9376,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="5" t="n">
         <v>159</v>
       </c>
@@ -9393,7 +9393,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="5" t="n">
         <v>160</v>
       </c>
@@ -9410,7 +9410,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="5" t="n">
         <v>161</v>
       </c>
@@ -9427,7 +9427,7 @@
         <v>995</v>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="5" t="n">
         <v>162</v>
       </c>
@@ -9444,7 +9444,7 @@
         <v>1007</v>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="5" t="n">
         <v>163</v>
       </c>

</xml_diff>

<commit_message>
Ingest approved entries (2026-08-28)
</commit_message>
<xml_diff>
--- a/data/Trump_Second_Term_Weekly_Tracker.xlsx
+++ b/data/Trump_Second_Term_Weekly_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$160</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$173</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1398" uniqueCount="1019">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="1055">
   <si>
     <t xml:space="preserve">Documented actions and policies of the second Trump administration reported as harmful by major news outlets, courts, and government data — Jan 20, 2025 through Jul 8, 2026. One row per event; weeks with multiple events have multiple rows; quiet weeks are skipped. This compiles critical coverage as requested; the administration and its supporters dispute many of these characterizations. See the Sources tab (matching Ref #) and verify details independently before citing.</t>
   </si>
@@ -1599,6 +1599,24 @@
     <t xml:space="preserve">Jul 14</t>
   </si>
   <si>
+    <t xml:space="preserve">Aug 17, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 21</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ref # matches the Source Ref column on the Weekly Timeline tab. URLs are provided where verified via current web results (mostly 2026 items). For 2025 items, outlet names and dates are given; searching the description text will locate the original coverage. Per your request the mix emphasizes CNN, Politico, MSNBC/MS NOW, NBC and independent outlets, alongside AP, Reuters, Guardian, NPR, CBS, ABC and court documents.</t>
   </si>
   <si>
@@ -3073,6 +3091,96 @@
   </si>
   <si>
     <t xml:space="preserve">Jul 14, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump ‘doesn’t have a plan’ on Iran: Voters in key Pennsylvania district upset with handling of war</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/meet-the-press/video/trump-doesn-t-have-a-plan-on-iran-voters-in-key-pennsylvania-district-upset-with-handling-of-war-268422725765</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Congresswoman says target of ICE operation in fatal Maine shooting wasn't up for removal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/congresswoman-target-ice-operation-fatal-maine-shooting-removal-135749324</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 18, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump administration moves ahead to end roadless rule on national forests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/trump-administration-moves-ahead-end-roadless-rule-national-135748769</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senator presses Hegseth, Caine for commitment to keep US military out of the midterm elections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/senator-presses-hegseth-caine-commitment-us-military-midterm-135745047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump tries to quiet his mass deportation campaign. Voters aren’t moving.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.politico.com/news/2026/08/19/poll-trump-deportations-voters-midterms-01041099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 19, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Has Trump no shame about all the money he has made since being in office? | Francine Prose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.theguardian.com/commentisfree/2026/aug/20/trump-money-earnings-billionaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 20, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From ‘predator’ to ‘conman’: how Michael Cohen has described Trump</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.theguardian.com/us-news/2026/aug/20/michael-cohen-donald-trump</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump talks about grass as he shows off White House renovations – video</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.theguardian.com/us-news/video/2026/aug/19/trump-talks-grass-white-house</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supreme Court allows Trump's ballroom construction to continue for now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.npr.org/2026/08/21/nx-s1-5935417/supreme-court-allows-trumps-ballroom-construction-to-continue-for-now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 21, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karoline Leavitt to work for Trump-affiliated super PAC after leaving White House</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/white-house/karoline-leavitt-work-trump-affiliated-super-pac-leaving-white-house-rcna593824</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navy discusses renaming aircraft carrier after Trump instead of heroic Black sailor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/trump-administration/navy-discusses-renaming-aircraft-carrier-trump-black-uss-doris-miller-rcna593667</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pentagon moves to fire publisher and editor of Stars and Stripes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cbsnews.com/news/stars-and-stripes-publisher-editor-separation-notices-pentagon/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Court says prosecutor who subpoenaed Letitia James was unlawfully appointed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cbsnews.com/news/appeals-court-john-sarcone-letitia-james-federal-prosecutor/</t>
   </si>
   <si>
     <t xml:space="preserve">Entries by category (live COUNTIF formulas against the Weekly Timeline tab)</t>
@@ -3554,7 +3662,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F165"/>
+  <dimension ref="A1:F173"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.01"/>
@@ -6743,47 +6851,189 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A161" s="4"/>
-      <c r="B161" s="4"/>
+      <c r="A161" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B161" s="4" t="s">
+        <v>525</v>
+      </c>
       <c r="C161" s="4"/>
       <c r="D161" s="4"/>
       <c r="E161" s="4"/>
-      <c r="F161" s="4"/>
+      <c r="F161" s="4" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A162" s="4"/>
-      <c r="B162" s="4"/>
+      <c r="A162" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B162" s="4" t="s">
+        <v>526</v>
+      </c>
       <c r="C162" s="4"/>
       <c r="D162" s="4"/>
       <c r="E162" s="4"/>
-      <c r="F162" s="4"/>
+      <c r="F162" s="4" t="n">
+        <v>160</v>
+      </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A163" s="4"/>
-      <c r="B163" s="4"/>
+      <c r="A163" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B163" s="4" t="s">
+        <v>526</v>
+      </c>
       <c r="C163" s="4"/>
       <c r="D163" s="4"/>
       <c r="E163" s="4"/>
-      <c r="F163" s="4"/>
+      <c r="F163" s="4" t="n">
+        <v>161</v>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A164" s="4"/>
-      <c r="B164" s="4"/>
+      <c r="A164" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B164" s="4" t="s">
+        <v>526</v>
+      </c>
       <c r="C164" s="4"/>
       <c r="D164" s="4"/>
       <c r="E164" s="4"/>
-      <c r="F164" s="4"/>
+      <c r="F164" s="4" t="n">
+        <v>162</v>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A165" s="4"/>
-      <c r="B165" s="4"/>
+      <c r="A165" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="B165" s="4" t="s">
+        <v>527</v>
+      </c>
       <c r="C165" s="4"/>
       <c r="D165" s="4"/>
       <c r="E165" s="4"/>
-      <c r="F165" s="4"/>
+      <c r="F165" s="4" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A166" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B166" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="C166" s="5"/>
+      <c r="D166" s="5"/>
+      <c r="E166" s="5"/>
+      <c r="F166" s="5" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A167" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B167" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="C167" s="5"/>
+      <c r="D167" s="5"/>
+      <c r="E167" s="5"/>
+      <c r="F167" s="5" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B168" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="C168" s="5"/>
+      <c r="D168" s="5"/>
+      <c r="E168" s="5"/>
+      <c r="F168" s="5" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C169" s="5"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B170" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C170" s="5"/>
+      <c r="D170" s="5"/>
+      <c r="E170" s="5"/>
+      <c r="F170" s="5" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B171" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C171" s="5"/>
+      <c r="D171" s="5"/>
+      <c r="E171" s="5"/>
+      <c r="F171" s="5" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B172" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C172" s="5"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+      <c r="F172" s="5" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="5" t="s">
+        <v>524</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="C173" s="5"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+      <c r="F173" s="5" t="n">
+        <v>171</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:F160"/>
+  <autoFilter ref="A2:F173"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -6803,7 +7053,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -6814,7 +7064,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6823,19 +7073,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6843,14 +7093,14 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6858,14 +7108,14 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6873,14 +7123,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6888,14 +7138,14 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6903,14 +7153,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6918,14 +7168,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6933,14 +7183,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6948,14 +7198,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6963,14 +7213,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6978,14 +7228,14 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6993,14 +7243,14 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7008,14 +7258,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7023,14 +7273,14 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7038,14 +7288,14 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7053,14 +7303,14 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7068,14 +7318,14 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
-        <v>574</v>
+        <v>580</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7083,14 +7333,14 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>576</v>
+        <v>582</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>577</v>
+        <v>583</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7098,14 +7348,14 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>578</v>
+        <v>584</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>579</v>
+        <v>585</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>580</v>
+        <v>586</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7113,14 +7363,14 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>581</v>
+        <v>587</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>582</v>
+        <v>588</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>583</v>
+        <v>589</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7128,14 +7378,14 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>584</v>
+        <v>590</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>585</v>
+        <v>591</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7143,14 +7393,14 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>587</v>
+        <v>593</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>588</v>
+        <v>594</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>589</v>
+        <v>595</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7158,14 +7408,14 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>590</v>
+        <v>596</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="s">
-        <v>592</v>
+        <v>598</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7173,14 +7423,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>593</v>
+        <v>599</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>594</v>
+        <v>600</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5" t="s">
-        <v>595</v>
+        <v>601</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7188,14 +7438,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7203,14 +7453,14 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7218,14 +7468,14 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>603</v>
+        <v>609</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
-        <v>604</v>
+        <v>610</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7233,14 +7483,14 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>605</v>
+        <v>611</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>606</v>
+        <v>612</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="s">
-        <v>607</v>
+        <v>613</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7248,14 +7498,14 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>608</v>
+        <v>614</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>609</v>
+        <v>615</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
-        <v>610</v>
+        <v>616</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7263,14 +7513,14 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>611</v>
+        <v>617</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>612</v>
+        <v>618</v>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7278,14 +7528,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>614</v>
+        <v>620</v>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="5" t="s">
-        <v>615</v>
+        <v>621</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7293,14 +7543,14 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>616</v>
+        <v>622</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>617</v>
+        <v>623</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="5" t="s">
-        <v>618</v>
+        <v>624</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7308,14 +7558,14 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>619</v>
+        <v>625</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="s">
-        <v>620</v>
+        <v>626</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7323,14 +7573,14 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>621</v>
+        <v>627</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>622</v>
+        <v>628</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="5" t="s">
-        <v>623</v>
+        <v>629</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7338,14 +7588,14 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>624</v>
+        <v>630</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>625</v>
+        <v>631</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="s">
-        <v>626</v>
+        <v>632</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7353,14 +7603,14 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7368,14 +7618,14 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="s">
-        <v>631</v>
+        <v>637</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7383,14 +7633,14 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7398,14 +7648,14 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="D40" s="5"/>
       <c r="E40" s="5" t="s">
-        <v>637</v>
+        <v>643</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7413,10 +7663,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="D41" s="5"/>
       <c r="E41" s="5" t="s">
@@ -7428,14 +7678,14 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7443,14 +7693,14 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="D43" s="5"/>
       <c r="E43" s="5" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7458,14 +7708,14 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D44" s="5"/>
       <c r="E44" s="5" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7473,14 +7723,14 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>649</v>
+        <v>655</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>650</v>
+        <v>656</v>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7488,14 +7738,14 @@
         <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="D46" s="5"/>
       <c r="E46" s="5" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7503,14 +7753,14 @@
         <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="D47" s="5"/>
       <c r="E47" s="5" t="s">
-        <v>657</v>
+        <v>663</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7518,14 +7768,14 @@
         <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>658</v>
+        <v>664</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>659</v>
+        <v>665</v>
       </c>
       <c r="D48" s="5"/>
       <c r="E48" s="5" t="s">
-        <v>660</v>
+        <v>666</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7533,14 +7783,14 @@
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>661</v>
+        <v>667</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>662</v>
+        <v>668</v>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="s">
-        <v>663</v>
+        <v>669</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7548,14 +7798,14 @@
         <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>664</v>
+        <v>670</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>665</v>
+        <v>671</v>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
-        <v>666</v>
+        <v>672</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7563,14 +7813,14 @@
         <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>667</v>
+        <v>673</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>668</v>
+        <v>674</v>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="s">
-        <v>669</v>
+        <v>675</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7578,14 +7828,14 @@
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>670</v>
+        <v>676</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>671</v>
+        <v>677</v>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="s">
-        <v>672</v>
+        <v>678</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7593,14 +7843,14 @@
         <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>674</v>
+        <v>680</v>
       </c>
       <c r="D53" s="5"/>
       <c r="E53" s="5" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7608,14 +7858,14 @@
         <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7623,14 +7873,14 @@
         <v>53</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D55" s="5"/>
       <c r="E55" s="5" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7638,14 +7888,14 @@
         <v>54</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="D56" s="5"/>
       <c r="E56" s="5" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7653,14 +7903,14 @@
         <v>55</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="D57" s="5"/>
       <c r="E57" s="5" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7668,14 +7918,14 @@
         <v>56</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7683,14 +7933,14 @@
         <v>57</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="D59" s="5"/>
       <c r="E59" s="5" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7698,14 +7948,14 @@
         <v>58</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>694</v>
+        <v>700</v>
       </c>
       <c r="D60" s="5"/>
       <c r="E60" s="5" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7713,14 +7963,14 @@
         <v>59</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="D61" s="5"/>
       <c r="E61" s="5" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7728,14 +7978,14 @@
         <v>60</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="D62" s="5"/>
       <c r="E62" s="5" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7743,14 +7993,14 @@
         <v>61</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="D63" s="5"/>
       <c r="E63" s="5" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7758,14 +8008,14 @@
         <v>62</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="D64" s="5"/>
       <c r="E64" s="5" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7773,14 +8023,14 @@
         <v>63</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7788,14 +8038,14 @@
         <v>64</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="D66" s="5"/>
       <c r="E66" s="5" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7803,14 +8053,14 @@
         <v>65</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="D67" s="5"/>
       <c r="E67" s="5" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7818,14 +8068,14 @@
         <v>66</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="D68" s="5"/>
       <c r="E68" s="5" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7833,14 +8083,14 @@
         <v>67</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="D69" s="5"/>
       <c r="E69" s="5" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7848,14 +8098,14 @@
         <v>68</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="D70" s="5"/>
       <c r="E70" s="5" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7863,14 +8113,14 @@
         <v>69</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="D71" s="5"/>
       <c r="E71" s="5" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7878,14 +8128,14 @@
         <v>70</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="D72" s="5"/>
       <c r="E72" s="5" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7893,14 +8143,14 @@
         <v>71</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="D73" s="5"/>
       <c r="E73" s="5" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7908,14 +8158,14 @@
         <v>72</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7923,14 +8173,14 @@
         <v>73</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>738</v>
+        <v>744</v>
       </c>
       <c r="D75" s="5"/>
       <c r="E75" s="5" t="s">
-        <v>739</v>
+        <v>745</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7938,14 +8188,14 @@
         <v>74</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>740</v>
+        <v>746</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>741</v>
+        <v>747</v>
       </c>
       <c r="D76" s="5"/>
       <c r="E76" s="5" t="s">
-        <v>742</v>
+        <v>748</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7953,14 +8203,14 @@
         <v>75</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>575</v>
+        <v>581</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>743</v>
+        <v>749</v>
       </c>
       <c r="D77" s="5"/>
       <c r="E77" s="5" t="s">
-        <v>744</v>
+        <v>750</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7968,14 +8218,14 @@
         <v>76</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>745</v>
+        <v>751</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>746</v>
+        <v>752</v>
       </c>
       <c r="D78" s="5"/>
       <c r="E78" s="5" t="s">
-        <v>747</v>
+        <v>753</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7983,14 +8233,14 @@
         <v>77</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>748</v>
+        <v>754</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>749</v>
+        <v>755</v>
       </c>
       <c r="D79" s="5"/>
       <c r="E79" s="5" t="s">
-        <v>750</v>
+        <v>756</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7998,14 +8248,14 @@
         <v>78</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>673</v>
+        <v>679</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>751</v>
+        <v>757</v>
       </c>
       <c r="D80" s="5"/>
       <c r="E80" s="5" t="s">
-        <v>752</v>
+        <v>758</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8013,14 +8263,14 @@
         <v>79</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="D81" s="5"/>
       <c r="E81" s="5" t="s">
-        <v>754</v>
+        <v>760</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8028,16 +8278,16 @@
         <v>80</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>755</v>
+        <v>761</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>756</v>
+        <v>762</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>757</v>
+        <v>763</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>758</v>
+        <v>764</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8045,16 +8295,16 @@
         <v>81</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>760</v>
+        <v>766</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>761</v>
+        <v>767</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8062,13 +8312,13 @@
         <v>82</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="E84" s="5" t="s">
         <v>297</v>
@@ -8079,13 +8329,13 @@
         <v>83</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>300</v>
@@ -8096,16 +8346,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8113,16 +8363,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8130,16 +8380,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>778</v>
+        <v>784</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>779</v>
+        <v>785</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8147,16 +8397,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="5" t="s">
-        <v>780</v>
+        <v>786</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>781</v>
+        <v>787</v>
       </c>
       <c r="D89" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>782</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>776</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8164,16 +8414,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>784</v>
+        <v>790</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>785</v>
+        <v>791</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8181,16 +8431,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>787</v>
+        <v>793</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>788</v>
+        <v>794</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>789</v>
+        <v>795</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>786</v>
+        <v>792</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8198,16 +8448,16 @@
         <v>90</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>790</v>
+        <v>796</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>791</v>
+        <v>797</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8215,16 +8465,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>793</v>
+        <v>799</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>794</v>
+        <v>800</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>795</v>
+        <v>801</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8232,16 +8482,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>796</v>
+        <v>802</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>797</v>
+        <v>803</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>798</v>
+        <v>804</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>799</v>
+        <v>805</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8249,16 +8499,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>800</v>
+        <v>806</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>801</v>
+        <v>807</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8266,16 +8516,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>804</v>
+        <v>810</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8283,16 +8533,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="C97" s="5" t="s">
-        <v>806</v>
+        <v>812</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>807</v>
+        <v>813</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>802</v>
+        <v>808</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8300,16 +8550,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>792</v>
+        <v>798</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8317,16 +8567,16 @@
         <v>97</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>812</v>
+        <v>818</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8334,16 +8584,16 @@
         <v>98</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>815</v>
+        <v>821</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8351,16 +8601,16 @@
         <v>99</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>817</v>
+        <v>823</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>819</v>
+        <v>825</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8368,16 +8618,16 @@
         <v>100</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>821</v>
+        <v>827</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>823</v>
+        <v>829</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8385,16 +8635,16 @@
         <v>101</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>825</v>
+        <v>831</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8402,13 +8652,13 @@
         <v>102</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>827</v>
+        <v>833</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>352</v>
@@ -8419,16 +8669,16 @@
         <v>103</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>831</v>
+        <v>837</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8436,16 +8686,16 @@
         <v>104</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>835</v>
+        <v>841</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8453,16 +8703,16 @@
         <v>105</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>838</v>
+        <v>844</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>840</v>
+        <v>846</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8470,16 +8720,16 @@
         <v>106</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>842</v>
+        <v>848</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8487,13 +8737,13 @@
         <v>107</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>845</v>
+        <v>851</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>846</v>
+        <v>852</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>368</v>
@@ -8504,13 +8754,13 @@
         <v>108</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>847</v>
+        <v>853</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>848</v>
+        <v>854</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>368</v>
@@ -8521,16 +8771,16 @@
         <v>109</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>849</v>
+        <v>855</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>850</v>
+        <v>856</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>851</v>
+        <v>857</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8538,16 +8788,16 @@
         <v>110</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>853</v>
+        <v>859</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>854</v>
+        <v>860</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8555,13 +8805,13 @@
         <v>111</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>855</v>
+        <v>861</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>856</v>
+        <v>862</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>382</v>
@@ -8572,16 +8822,16 @@
         <v>112</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>857</v>
+        <v>863</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>858</v>
+        <v>864</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>859</v>
+        <v>865</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8589,16 +8839,16 @@
         <v>113</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>861</v>
+        <v>867</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>862</v>
+        <v>868</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8606,16 +8856,16 @@
         <v>114</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>864</v>
+        <v>870</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>865</v>
+        <v>871</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>863</v>
+        <v>869</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8623,16 +8873,16 @@
         <v>115</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>866</v>
+        <v>872</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>867</v>
+        <v>873</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>868</v>
+        <v>874</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>869</v>
+        <v>875</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8640,13 +8890,13 @@
         <v>116</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>870</v>
+        <v>876</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>871</v>
+        <v>877</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>396</v>
@@ -8657,16 +8907,16 @@
         <v>117</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>872</v>
+        <v>878</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>873</v>
+        <v>879</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>874</v>
+        <v>880</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>875</v>
+        <v>881</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8674,16 +8924,16 @@
         <v>118</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>876</v>
+        <v>882</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>877</v>
+        <v>883</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>878</v>
+        <v>884</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8691,16 +8941,16 @@
         <v>119</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>879</v>
+        <v>885</v>
       </c>
       <c r="C121" s="5" t="s">
-        <v>880</v>
+        <v>886</v>
       </c>
       <c r="D121" s="6" t="s">
+        <v>887</v>
+      </c>
+      <c r="E121" s="5" t="s">
         <v>881</v>
-      </c>
-      <c r="E121" s="5" t="s">
-        <v>875</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8708,16 +8958,16 @@
         <v>120</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>882</v>
+        <v>888</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>883</v>
+        <v>889</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>884</v>
+        <v>890</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>885</v>
+        <v>891</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8725,13 +8975,13 @@
         <v>121</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>783</v>
+        <v>789</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>886</v>
+        <v>892</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>887</v>
+        <v>893</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>409</v>
@@ -8742,13 +8992,13 @@
         <v>122</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>888</v>
+        <v>894</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>889</v>
+        <v>895</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>409</v>
@@ -8759,16 +9009,16 @@
         <v>123</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>890</v>
+        <v>896</v>
       </c>
       <c r="D125" s="6" t="s">
-        <v>891</v>
+        <v>897</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8776,16 +9026,16 @@
         <v>124</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>893</v>
+        <v>899</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>894</v>
+        <v>900</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>895</v>
+        <v>901</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>892</v>
+        <v>898</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8793,16 +9043,16 @@
         <v>125</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>829</v>
+        <v>835</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>896</v>
+        <v>902</v>
       </c>
       <c r="D127" s="6" t="s">
-        <v>897</v>
+        <v>903</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>898</v>
+        <v>904</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8810,16 +9060,16 @@
         <v>126</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>899</v>
+        <v>905</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>900</v>
+        <v>906</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>902</v>
+        <v>908</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8827,16 +9077,16 @@
         <v>127</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>903</v>
+        <v>909</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>904</v>
+        <v>910</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>906</v>
+        <v>912</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8844,16 +9094,16 @@
         <v>128</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>907</v>
+        <v>913</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>908</v>
+        <v>914</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>909</v>
+        <v>915</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8861,13 +9111,13 @@
         <v>129</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>910</v>
+        <v>916</v>
       </c>
       <c r="C131" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="D131" s="6" t="s">
         <v>911</v>
-      </c>
-      <c r="D131" s="6" t="s">
-        <v>905</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>434</v>
@@ -8878,16 +9128,16 @@
         <v>130</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>912</v>
+        <v>918</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>913</v>
+        <v>919</v>
       </c>
       <c r="D132" s="6" t="s">
-        <v>914</v>
+        <v>920</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8895,16 +9145,16 @@
         <v>131</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>916</v>
+        <v>922</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>917</v>
+        <v>923</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>918</v>
+        <v>924</v>
       </c>
       <c r="E133" s="5" t="s">
-        <v>915</v>
+        <v>921</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8912,16 +9162,16 @@
         <v>132</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>919</v>
+        <v>925</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>920</v>
+        <v>926</v>
       </c>
       <c r="D134" s="6" t="s">
-        <v>921</v>
+        <v>927</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>922</v>
+        <v>928</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8929,16 +9179,16 @@
         <v>133</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>923</v>
+        <v>929</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>924</v>
+        <v>930</v>
       </c>
       <c r="D135" s="6" t="s">
-        <v>925</v>
+        <v>931</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>926</v>
+        <v>932</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8946,13 +9196,13 @@
         <v>134</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>927</v>
+        <v>933</v>
       </c>
       <c r="D136" s="6" t="s">
-        <v>928</v>
+        <v>934</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>451</v>
@@ -8963,13 +9213,13 @@
         <v>135</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>929</v>
+        <v>935</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>930</v>
+        <v>936</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>931</v>
+        <v>937</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>451</v>
@@ -8980,16 +9230,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>932</v>
+        <v>938</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>933</v>
+        <v>939</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>934</v>
+        <v>940</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>935</v>
+        <v>941</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8997,16 +9247,16 @@
         <v>137</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>936</v>
+        <v>942</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>937</v>
+        <v>943</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>938</v>
+        <v>944</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>939</v>
+        <v>945</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9014,13 +9264,13 @@
         <v>138</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>805</v>
+        <v>811</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>940</v>
+        <v>946</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>941</v>
+        <v>947</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>463</v>
@@ -9031,16 +9281,16 @@
         <v>139</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>942</v>
+        <v>948</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>943</v>
+        <v>949</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>944</v>
+        <v>950</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9048,16 +9298,16 @@
         <v>140</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>945</v>
+        <v>951</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>948</v>
+        <v>954</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9065,13 +9315,13 @@
         <v>141</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>949</v>
+        <v>955</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>950</v>
+        <v>956</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>472</v>
@@ -9082,16 +9332,16 @@
         <v>142</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>951</v>
+        <v>957</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>952</v>
+        <v>958</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>953</v>
+        <v>959</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>954</v>
+        <v>960</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9099,13 +9349,13 @@
         <v>143</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>955</v>
+        <v>961</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>956</v>
+        <v>962</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>479</v>
@@ -9116,16 +9366,16 @@
         <v>144</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>957</v>
+        <v>963</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>958</v>
+        <v>964</v>
       </c>
       <c r="E146" s="5" t="s">
-        <v>959</v>
+        <v>965</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9133,16 +9383,16 @@
         <v>145</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>960</v>
+        <v>966</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>961</v>
+        <v>967</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>962</v>
+        <v>968</v>
       </c>
       <c r="E147" s="5" t="s">
-        <v>963</v>
+        <v>969</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9150,16 +9400,16 @@
         <v>146</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>964</v>
+        <v>970</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>965</v>
+        <v>971</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>966</v>
+        <v>972</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>967</v>
+        <v>973</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9167,13 +9417,13 @@
         <v>147</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>968</v>
+        <v>974</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>969</v>
+        <v>975</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>901</v>
+        <v>907</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>492</v>
@@ -9184,13 +9434,13 @@
         <v>148</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>970</v>
+        <v>976</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>905</v>
+        <v>911</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>492</v>
@@ -9201,16 +9451,16 @@
         <v>149</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>973</v>
+        <v>979</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9218,16 +9468,16 @@
         <v>150</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>972</v>
+        <v>978</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>976</v>
+        <v>982</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>974</v>
+        <v>980</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>975</v>
+        <v>981</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9235,16 +9485,16 @@
         <v>151</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>978</v>
+        <v>984</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9252,16 +9502,16 @@
         <v>152</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>977</v>
+        <v>983</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>981</v>
+        <v>987</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>979</v>
+        <v>985</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>980</v>
+        <v>986</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9269,16 +9519,16 @@
         <v>153</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>982</v>
+        <v>988</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>983</v>
+        <v>989</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>984</v>
+        <v>990</v>
       </c>
       <c r="E155" s="5" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9286,16 +9536,16 @@
         <v>154</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>986</v>
+        <v>992</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>987</v>
+        <v>993</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>985</v>
+        <v>991</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9303,14 +9553,14 @@
         <v>155</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>988</v>
+        <v>994</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>989</v>
+        <v>995</v>
       </c>
       <c r="D157" s="5"/>
       <c r="E157" s="5" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9318,16 +9568,16 @@
         <v>156</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>992</v>
+        <v>998</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>993</v>
+        <v>999</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>990</v>
+        <v>996</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9335,16 +9585,16 @@
         <v>157</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>994</v>
+        <v>1000</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>995</v>
+        <v>1001</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9352,16 +9602,16 @@
         <v>158</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>777</v>
+        <v>783</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>997</v>
+        <v>1003</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>998</v>
+        <v>1004</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9369,16 +9619,16 @@
         <v>159</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>833</v>
+        <v>839</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>999</v>
+        <v>1005</v>
       </c>
       <c r="D161" s="6" t="s">
-        <v>1000</v>
+        <v>1006</v>
       </c>
       <c r="E161" s="5" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9386,16 +9636,16 @@
         <v>160</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="C162" s="5" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D162" s="6" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E162" s="5" t="s">
         <v>1002</v>
-      </c>
-      <c r="D162" s="6" t="s">
-        <v>1003</v>
-      </c>
-      <c r="E162" s="5" t="s">
-        <v>996</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9403,16 +9653,16 @@
         <v>161</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>1004</v>
+        <v>1010</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>1005</v>
+        <v>1011</v>
       </c>
       <c r="E163" s="5" t="s">
-        <v>996</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9420,16 +9670,16 @@
         <v>162</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
       <c r="C164" s="5" t="s">
-        <v>1006</v>
+        <v>1012</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>1007</v>
+        <v>1013</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>1008</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9437,50 +9687,271 @@
         <v>163</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>638</v>
+        <v>644</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>1009</v>
+        <v>1015</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>1010</v>
+        <v>1016</v>
       </c>
       <c r="E165" s="5" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="166" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="5" t="n">
         <v>157</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>1001</v>
+        <v>1007</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>1011</v>
+        <v>1017</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>1012</v>
+        <v>1018</v>
       </c>
       <c r="E166" s="5" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="5" t="n">
         <v>158</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>860</v>
+        <v>866</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="D167" s="6" t="s">
-        <v>1014</v>
+        <v>1020</v>
       </c>
       <c r="E167" s="5" t="s">
-        <v>1015</v>
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="168" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A168" s="5" t="n">
+        <v>159</v>
+      </c>
+      <c r="B168" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="C168" s="5" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D168" s="6" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E168" s="5" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="169" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A169" s="5" t="n">
+        <v>160</v>
+      </c>
+      <c r="B169" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="C169" s="5" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D169" s="6" t="s">
+        <v>1025</v>
+      </c>
+      <c r="E169" s="5" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A170" s="5" t="n">
+        <v>161</v>
+      </c>
+      <c r="B170" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="C170" s="5" t="s">
+        <v>1027</v>
+      </c>
+      <c r="D170" s="6" t="s">
+        <v>1028</v>
+      </c>
+      <c r="E170" s="5" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="171" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A171" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="B171" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="C171" s="5" t="s">
+        <v>1029</v>
+      </c>
+      <c r="D171" s="6" t="s">
+        <v>1030</v>
+      </c>
+      <c r="E171" s="5" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A172" s="5" t="n">
+        <v>163</v>
+      </c>
+      <c r="B172" s="5" t="s">
+        <v>789</v>
+      </c>
+      <c r="C172" s="5" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D172" s="6" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E172" s="5" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="173" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A173" s="5" t="n">
+        <v>164</v>
+      </c>
+      <c r="B173" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="C173" s="5" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D173" s="6" t="s">
+        <v>1035</v>
+      </c>
+      <c r="E173" s="5" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A174" s="5" t="n">
+        <v>165</v>
+      </c>
+      <c r="B174" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="C174" s="5" t="s">
+        <v>1037</v>
+      </c>
+      <c r="D174" s="6" t="s">
+        <v>1038</v>
+      </c>
+      <c r="E174" s="5" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A175" s="5" t="n">
+        <v>166</v>
+      </c>
+      <c r="B175" s="5" t="s">
+        <v>783</v>
+      </c>
+      <c r="C175" s="5" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D175" s="6" t="s">
+        <v>1040</v>
+      </c>
+      <c r="E175" s="5" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A176" s="5" t="n">
+        <v>167</v>
+      </c>
+      <c r="B176" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="C176" s="5" t="s">
+        <v>1041</v>
+      </c>
+      <c r="D176" s="6" t="s">
+        <v>1042</v>
+      </c>
+      <c r="E176" s="5" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A177" s="5" t="n">
+        <v>168</v>
+      </c>
+      <c r="B177" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D177" s="6" t="s">
+        <v>1045</v>
+      </c>
+      <c r="E177" s="5" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A178" s="5" t="n">
+        <v>169</v>
+      </c>
+      <c r="B178" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D178" s="6" t="s">
+        <v>1047</v>
+      </c>
+      <c r="E178" s="5" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A179" s="5" t="n">
+        <v>170</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>866</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D179" s="6" t="s">
+        <v>1049</v>
+      </c>
+      <c r="E179" s="5" t="s">
+        <v>1043</v>
+      </c>
+    </row>
+    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A180" s="5" t="n">
+        <v>171</v>
+      </c>
+      <c r="B180" s="5" t="s">
+        <v>866</v>
+      </c>
+      <c r="C180" s="5" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D180" s="6" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E180" s="5" t="s">
+        <v>1043</v>
       </c>
     </row>
   </sheetData>
@@ -9573,6 +10044,19 @@
     <hyperlink ref="D165" r:id="rId83" display="https://www.nbcnews.com/politics/justice-department/judge-grants-doj-request-toss-remaining-jan-6-convictions-proud-boys-rcna385952"/>
     <hyperlink ref="D166" r:id="rId84" display="https://www.pbs.org/newshour/nation/ice-shot-and-killed-a-colombian-man-in-maine-this-is-the-2nd-time-in-a-week-the-agency-used-deadly-force"/>
     <hyperlink ref="D167" r:id="rId85" display="https://www.cbsnews.com/news/iran-military-action-formally-restarted-trump-lawmakers-war-powers/"/>
+    <hyperlink ref="D168" r:id="rId86" display="https://www.nbcnews.com/meet-the-press/video/trump-doesn-t-have-a-plan-on-iran-voters-in-key-pennsylvania-district-upset-with-handling-of-war-268422725765"/>
+    <hyperlink ref="D169" r:id="rId87" display="https://abcnews.com/Politics/wireStory/congresswoman-target-ice-operation-fatal-maine-shooting-removal-135749324"/>
+    <hyperlink ref="D170" r:id="rId88" display="https://abcnews.com/Politics/wireStory/trump-administration-moves-ahead-end-roadless-rule-national-135748769"/>
+    <hyperlink ref="D171" r:id="rId89" display="https://abcnews.com/Politics/wireStory/senator-presses-hegseth-caine-commitment-us-military-midterm-135745047"/>
+    <hyperlink ref="D172" r:id="rId90" display="https://www.politico.com/news/2026/08/19/poll-trump-deportations-voters-midterms-01041099"/>
+    <hyperlink ref="D173" r:id="rId91" display="https://www.theguardian.com/commentisfree/2026/aug/20/trump-money-earnings-billionaires"/>
+    <hyperlink ref="D174" r:id="rId92" display="https://www.theguardian.com/us-news/2026/aug/20/michael-cohen-donald-trump"/>
+    <hyperlink ref="D175" r:id="rId93" display="https://www.theguardian.com/us-news/video/2026/aug/19/trump-talks-grass-white-house"/>
+    <hyperlink ref="D176" r:id="rId94" display="https://www.npr.org/2026/08/21/nx-s1-5935417/supreme-court-allows-trumps-ballroom-construction-to-continue-for-now"/>
+    <hyperlink ref="D177" r:id="rId95" display="https://www.nbcnews.com/politics/white-house/karoline-leavitt-work-trump-affiliated-super-pac-leaving-white-house-rcna593824"/>
+    <hyperlink ref="D178" r:id="rId96" display="https://www.nbcnews.com/politics/trump-administration/navy-discusses-renaming-aircraft-carrier-trump-black-uss-doris-miller-rcna593667"/>
+    <hyperlink ref="D179" r:id="rId97" display="https://www.cbsnews.com/news/stars-and-stripes-publisher-editor-separation-notices-pentagon/"/>
+    <hyperlink ref="D180" r:id="rId98" display="https://www.cbsnews.com/news/appeals-court-john-sarcone-letitia-james-federal-prosecutor/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -9598,7 +10082,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>1016</v>
+        <v>1052</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -9607,7 +10091,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1017</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9765,7 +10249,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1018</v>
+        <v>1054</v>
       </c>
       <c r="B20" s="10" t="n">
         <f aca="false">SUM(B3:B19)</f>

</xml_diff>

<commit_message>
Ingest approved entries (2026-08-30)
</commit_message>
<xml_diff>
--- a/data/Trump_Second_Term_Weekly_Tracker.xlsx
+++ b/data/Trump_Second_Term_Weekly_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$213</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$222</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1716" uniqueCount="1165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1778" uniqueCount="1190">
   <si>
     <t xml:space="preserve">Documented actions and policies of the second Trump administration reported as harmful by major news outlets, courts, and government data — Jan 20, 2025 through Jul 8, 2026. One row per event; weeks with multiple events have multiple rows; quiet weeks are skipped. This compiles critical coverage as requested; the administration and its supporters dispute many of these characterizations. See the Sources tab (matching Ref #) and verify details independently before citing.</t>
   </si>
@@ -1668,6 +1668,18 @@
     <t xml:space="preserve">Jul 17</t>
   </si>
   <si>
+    <t xml:space="preserve">Aug 24, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 28</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ref # matches the Source Ref column on the Weekly Timeline tab. URLs are provided where verified via current web results (mostly 2026 items). For 2025 items, outlet names and dates are given; searching the description text will locate the original coverage. Per your request the mix emphasizes CNN, Politico, MSNBC/MS NOW, NBC and independent outlets, alongside AP, Reuters, Guardian, NPR, CBS, ABC and court documents.</t>
   </si>
   <si>
@@ -3511,6 +3523,69 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.pbs.org/newshour/show/trump-tries-to-undermine-trust-in-elections-but-documents-dont-support-his-claims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Democratic states file new lawsuit seeking to block Trump’s order limiting mail voting in midterms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/democratic-states-file-new-lawsuit-seeking-block-trumps-135974009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 26, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump signs executive order to rename Lake Ontario as ‘Lake America’</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/trump-administration/trump-orders-lake-ontario-renamed-lake-america-canada-trade-war-rcna594750</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 27, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group of Democratic senators calls on ICE to cancel plan to buy electric shock gloves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/group-democratic-senators-calls-ice-cancel-plan-buy-136008188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US goals have shifted after 6 months of Iran war. The Strait of Hormuz is now a top concern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/us-goals-shifted-after-6-months-iran-war-135995683</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan. 6 rioters pursue new path for payments from Trump administration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pbs.org/newshour/show/jan-6-rioters-pursue-new-path-for-payments-from-trump-administration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump administration proposal would allow federal grants to be terminated on a whim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.npr.org/2026/08/28/nx-s1-5943238/trump-administration-proposal-would-allow-federal-grants-to-be-terminated-on-a-whim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aug 28, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump signs order to create space-focused military academy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/trump-administration/trump-space-academy-nasa-military-rcna594870</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How did Trump get so rich? | Politics Weekly America</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.theguardian.com/politics/video/2026/aug/27/how-did-trump-get-so-rich-politics-weekly-america</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U.S. targets Egyptian bank's UAE branches under new push for Iran's economic isolation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pbs.org/newshour/world/u-s-targets-egyptian-banks-uae-branches-under-new-push-for-irans-economic-isolation</t>
   </si>
   <si>
     <t xml:space="preserve">Entries by category (live COUNTIF formulas against the Weekly Timeline tab)</t>
@@ -3992,7 +4067,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F213"/>
+  <dimension ref="A1:F222"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.01"/>
@@ -7810,7 +7885,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="4" t="s">
         <v>521</v>
       </c>
@@ -7824,7 +7899,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="4" t="s">
         <v>521</v>
       </c>
@@ -7838,7 +7913,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="4" t="s">
         <v>521</v>
       </c>
@@ -7852,7 +7927,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="4" t="s">
         <v>521</v>
       </c>
@@ -7866,7 +7941,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="4" t="s">
         <v>521</v>
       </c>
@@ -7880,7 +7955,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="4" t="s">
         <v>521</v>
       </c>
@@ -7894,7 +7969,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="4" t="s">
         <v>521</v>
       </c>
@@ -7908,7 +7983,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="4" t="s">
         <v>521</v>
       </c>
@@ -7922,8 +7997,150 @@
         <v>211</v>
       </c>
     </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A214" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B214" s="5" t="s">
+        <v>548</v>
+      </c>
+      <c r="C214" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D214" s="5"/>
+      <c r="E214" s="5"/>
+      <c r="F214" s="5" t="n">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A215" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B215" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C215" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D215" s="5"/>
+      <c r="E215" s="5"/>
+      <c r="F215" s="5" t="n">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A216" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B216" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C216" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="D216" s="5"/>
+      <c r="E216" s="5"/>
+      <c r="F216" s="5" t="n">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A217" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D217" s="5"/>
+      <c r="E217" s="5"/>
+      <c r="F217" s="5" t="n">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A218" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B218" s="5" t="s">
+        <v>549</v>
+      </c>
+      <c r="C218" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D218" s="5"/>
+      <c r="E218" s="5"/>
+      <c r="F218" s="5" t="n">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A219" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B219" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C219" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D219" s="5"/>
+      <c r="E219" s="5"/>
+      <c r="F219" s="5" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A220" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B220" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C220" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D220" s="5"/>
+      <c r="E220" s="5"/>
+      <c r="F220" s="5" t="n">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B221" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C221" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D221" s="5"/>
+      <c r="E221" s="5"/>
+      <c r="F221" s="5" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B222" s="5" t="s">
+        <v>550</v>
+      </c>
+      <c r="C222" s="5"/>
+      <c r="D222" s="5"/>
+      <c r="E222" s="5"/>
+      <c r="F222" s="5" t="n">
+        <v>220</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:F213"/>
+  <autoFilter ref="A2:F222"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -7943,7 +8160,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E220"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -7954,7 +8171,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7963,19 +8180,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7983,14 +8200,14 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7998,14 +8215,14 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8013,14 +8230,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8028,14 +8245,14 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8043,14 +8260,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8058,14 +8275,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8073,14 +8290,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8088,14 +8305,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8103,14 +8320,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8118,14 +8335,14 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8133,14 +8350,14 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8148,14 +8365,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8163,14 +8380,14 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8178,14 +8395,14 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8193,14 +8410,14 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8208,14 +8425,14 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8223,14 +8440,14 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8238,14 +8455,14 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8253,14 +8470,14 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8268,14 +8485,14 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8283,14 +8500,14 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8298,14 +8515,14 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8313,14 +8530,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8328,14 +8545,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8343,14 +8560,14 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8358,14 +8575,14 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8373,14 +8590,14 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8388,14 +8605,14 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8403,14 +8620,14 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8418,14 +8635,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="5" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8433,14 +8650,14 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="5" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8448,14 +8665,14 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8463,14 +8680,14 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="5" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8478,14 +8695,14 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8493,14 +8710,14 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8508,14 +8725,14 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8523,14 +8740,14 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8538,14 +8755,14 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="D40" s="5"/>
       <c r="E40" s="5" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8553,10 +8770,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="D41" s="5"/>
       <c r="E41" s="5" t="s">
@@ -8568,14 +8785,14 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8583,14 +8800,14 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="D43" s="5"/>
       <c r="E43" s="5" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8598,14 +8815,14 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="D44" s="5"/>
       <c r="E44" s="5" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8613,14 +8830,14 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8628,14 +8845,14 @@
         <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="D46" s="5"/>
       <c r="E46" s="5" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8643,14 +8860,14 @@
         <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="D47" s="5"/>
       <c r="E47" s="5" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8658,14 +8875,14 @@
         <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="D48" s="5"/>
       <c r="E48" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8673,14 +8890,14 @@
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8688,14 +8905,14 @@
         <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8703,14 +8920,14 @@
         <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8718,14 +8935,14 @@
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8733,14 +8950,14 @@
         <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D53" s="5"/>
       <c r="E53" s="5" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8748,14 +8965,14 @@
         <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8763,14 +8980,14 @@
         <v>53</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="D55" s="5"/>
       <c r="E55" s="5" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8778,14 +8995,14 @@
         <v>54</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="D56" s="5"/>
       <c r="E56" s="5" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8793,14 +9010,14 @@
         <v>55</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="D57" s="5"/>
       <c r="E57" s="5" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8808,14 +9025,14 @@
         <v>56</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8823,14 +9040,14 @@
         <v>57</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="D59" s="5"/>
       <c r="E59" s="5" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8838,14 +9055,14 @@
         <v>58</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="D60" s="5"/>
       <c r="E60" s="5" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8853,14 +9070,14 @@
         <v>59</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="D61" s="5"/>
       <c r="E61" s="5" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8868,14 +9085,14 @@
         <v>60</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="D62" s="5"/>
       <c r="E62" s="5" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8883,14 +9100,14 @@
         <v>61</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="D63" s="5"/>
       <c r="E63" s="5" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8898,14 +9115,14 @@
         <v>62</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="D64" s="5"/>
       <c r="E64" s="5" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8913,14 +9130,14 @@
         <v>63</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8928,14 +9145,14 @@
         <v>64</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="D66" s="5"/>
       <c r="E66" s="5" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8943,14 +9160,14 @@
         <v>65</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="D67" s="5"/>
       <c r="E67" s="5" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8958,14 +9175,14 @@
         <v>66</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="D68" s="5"/>
       <c r="E68" s="5" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8973,14 +9190,14 @@
         <v>67</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D69" s="5"/>
       <c r="E69" s="5" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8988,14 +9205,14 @@
         <v>68</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="D70" s="5"/>
       <c r="E70" s="5" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9003,14 +9220,14 @@
         <v>69</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="D71" s="5"/>
       <c r="E71" s="5" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9018,14 +9235,14 @@
         <v>70</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="D72" s="5"/>
       <c r="E72" s="5" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9033,14 +9250,14 @@
         <v>71</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="D73" s="5"/>
       <c r="E73" s="5" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9048,14 +9265,14 @@
         <v>72</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9063,14 +9280,14 @@
         <v>73</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="D75" s="5"/>
       <c r="E75" s="5" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9078,14 +9295,14 @@
         <v>74</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D76" s="5"/>
       <c r="E76" s="5" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9093,14 +9310,14 @@
         <v>75</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="D77" s="5"/>
       <c r="E77" s="5" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9108,14 +9325,14 @@
         <v>76</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="D78" s="5"/>
       <c r="E78" s="5" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9123,14 +9340,14 @@
         <v>77</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="D79" s="5"/>
       <c r="E79" s="5" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9138,14 +9355,14 @@
         <v>78</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="D80" s="5"/>
       <c r="E80" s="5" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9153,14 +9370,14 @@
         <v>79</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="D81" s="5"/>
       <c r="E81" s="5" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9168,16 +9385,16 @@
         <v>80</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9185,16 +9402,16 @@
         <v>81</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9202,13 +9419,13 @@
         <v>82</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="E84" s="5" t="s">
         <v>297</v>
@@ -9219,13 +9436,13 @@
         <v>83</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>300</v>
@@ -9236,16 +9453,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9253,16 +9470,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9270,16 +9487,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9287,16 +9504,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>803</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>804</v>
-      </c>
-      <c r="D89" s="6" t="s">
-        <v>805</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>799</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9304,16 +9521,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>807</v>
+        <v>811</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>808</v>
+        <v>812</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9321,16 +9538,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>809</v>
+        <v>813</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9338,16 +9555,16 @@
         <v>90</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9355,16 +9572,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9372,16 +9589,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9389,16 +9606,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9406,16 +9623,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9423,16 +9640,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="C97" s="5" t="s">
+        <v>833</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>834</v>
+      </c>
+      <c r="E97" s="5" t="s">
         <v>829</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>830</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>825</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9440,16 +9657,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9457,16 +9674,16 @@
         <v>97</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>834</v>
+        <v>838</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9474,16 +9691,16 @@
         <v>98</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9491,16 +9708,16 @@
         <v>99</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9508,16 +9725,16 @@
         <v>100</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9525,16 +9742,16 @@
         <v>101</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9542,13 +9759,13 @@
         <v>102</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>352</v>
@@ -9559,16 +9776,16 @@
         <v>103</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9576,16 +9793,16 @@
         <v>104</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9593,16 +9810,16 @@
         <v>105</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9610,16 +9827,16 @@
         <v>106</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9627,13 +9844,13 @@
         <v>107</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>368</v>
@@ -9644,13 +9861,13 @@
         <v>108</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>368</v>
@@ -9661,16 +9878,16 @@
         <v>109</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9678,16 +9895,16 @@
         <v>110</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9695,13 +9912,13 @@
         <v>111</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>382</v>
@@ -9712,16 +9929,16 @@
         <v>112</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9729,16 +9946,16 @@
         <v>113</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9746,16 +9963,16 @@
         <v>114</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9763,16 +9980,16 @@
         <v>115</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9780,13 +9997,13 @@
         <v>116</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>396</v>
@@ -9797,16 +10014,16 @@
         <v>117</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9814,16 +10031,16 @@
         <v>118</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9831,16 +10048,16 @@
         <v>119</v>
       </c>
       <c r="B121" s="5" t="s">
+        <v>906</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>907</v>
+      </c>
+      <c r="D121" s="6" t="s">
+        <v>908</v>
+      </c>
+      <c r="E121" s="5" t="s">
         <v>902</v>
-      </c>
-      <c r="C121" s="5" t="s">
-        <v>903</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>904</v>
-      </c>
-      <c r="E121" s="5" t="s">
-        <v>898</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9848,16 +10065,16 @@
         <v>120</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9865,13 +10082,13 @@
         <v>121</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>409</v>
@@ -9882,13 +10099,13 @@
         <v>122</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>409</v>
@@ -9899,16 +10116,16 @@
         <v>123</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="D125" s="6" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9916,16 +10133,16 @@
         <v>124</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9933,16 +10150,16 @@
         <v>125</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="D127" s="6" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9950,16 +10167,16 @@
         <v>126</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9967,16 +10184,16 @@
         <v>127</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9984,16 +10201,16 @@
         <v>128</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10001,13 +10218,13 @@
         <v>129</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="D131" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>434</v>
@@ -10018,16 +10235,16 @@
         <v>130</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
       <c r="D132" s="6" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10035,16 +10252,16 @@
         <v>131</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="E133" s="5" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10052,16 +10269,16 @@
         <v>132</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="D134" s="6" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10069,16 +10286,16 @@
         <v>133</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="D135" s="6" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10086,13 +10303,13 @@
         <v>134</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="D136" s="6" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>451</v>
@@ -10103,13 +10320,13 @@
         <v>135</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>451</v>
@@ -10120,16 +10337,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10137,16 +10354,16 @@
         <v>137</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>959</v>
+        <v>963</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10154,13 +10371,13 @@
         <v>138</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>463</v>
@@ -10171,16 +10388,16 @@
         <v>139</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10188,16 +10405,16 @@
         <v>140</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10205,13 +10422,13 @@
         <v>141</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>472</v>
@@ -10222,16 +10439,16 @@
         <v>142</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10239,13 +10456,13 @@
         <v>143</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>479</v>
@@ -10256,16 +10473,16 @@
         <v>144</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
       <c r="E146" s="5" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10273,16 +10490,16 @@
         <v>145</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="E147" s="5" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10290,16 +10507,16 @@
         <v>146</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>987</v>
+        <v>991</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>990</v>
+        <v>994</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10307,13 +10524,13 @@
         <v>147</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>492</v>
@@ -10324,13 +10541,13 @@
         <v>148</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>993</v>
+        <v>997</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>492</v>
@@ -10341,16 +10558,16 @@
         <v>149</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>996</v>
+        <v>1000</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>997</v>
+        <v>1001</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10358,16 +10575,16 @@
         <v>150</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>997</v>
+        <v>1001</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10375,16 +10592,16 @@
         <v>151</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10392,16 +10609,16 @@
         <v>152</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10409,16 +10626,16 @@
         <v>153</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="E155" s="5" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10426,16 +10643,16 @@
         <v>154</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>833</v>
+        <v>837</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10443,14 +10660,14 @@
         <v>155</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
       <c r="D157" s="5"/>
       <c r="E157" s="5" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10458,16 +10675,16 @@
         <v>156</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>1015</v>
+        <v>1019</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10475,16 +10692,16 @@
         <v>157</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10492,16 +10709,16 @@
         <v>158</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10509,16 +10726,16 @@
         <v>159</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="D161" s="6" t="s">
+        <v>1027</v>
+      </c>
+      <c r="E161" s="5" t="s">
         <v>1023</v>
-      </c>
-      <c r="E161" s="5" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10526,16 +10743,16 @@
         <v>160</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="E162" s="5" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10543,16 +10760,16 @@
         <v>161</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>1027</v>
+        <v>1031</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="E163" s="5" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10560,16 +10777,16 @@
         <v>162</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C164" s="5" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>1030</v>
+        <v>1034</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10577,16 +10794,16 @@
         <v>163</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="E165" s="5" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10594,13 +10811,13 @@
         <v>157</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
       <c r="E166" s="5" t="s">
         <v>521</v>
@@ -10611,16 +10828,16 @@
         <v>158</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="D167" s="6" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="E167" s="5" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10628,13 +10845,13 @@
         <v>159</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="D168" s="6" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="E168" s="5" t="s">
         <v>524</v>
@@ -10645,16 +10862,16 @@
         <v>160</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="D169" s="6" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
       <c r="E169" s="5" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10662,16 +10879,16 @@
         <v>161</v>
       </c>
       <c r="B170" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>1044</v>
+        <v>1048</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>1045</v>
+        <v>1049</v>
       </c>
       <c r="E170" s="5" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10679,16 +10896,16 @@
         <v>162</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>1046</v>
+        <v>1050</v>
       </c>
       <c r="D171" s="6" t="s">
+        <v>1051</v>
+      </c>
+      <c r="E171" s="5" t="s">
         <v>1047</v>
-      </c>
-      <c r="E171" s="5" t="s">
-        <v>1043</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10696,16 +10913,16 @@
         <v>163</v>
       </c>
       <c r="B172" s="5" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="D172" s="6" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="E172" s="5" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10713,16 +10930,16 @@
         <v>164</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>1051</v>
+        <v>1055</v>
       </c>
       <c r="D173" s="6" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="E173" s="5" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10730,16 +10947,16 @@
         <v>165</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
       <c r="D174" s="6" t="s">
-        <v>1055</v>
+        <v>1059</v>
       </c>
       <c r="E174" s="5" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10747,16 +10964,16 @@
         <v>166</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="D175" s="6" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E175" s="5" t="s">
         <v>1057</v>
-      </c>
-      <c r="E175" s="5" t="s">
-        <v>1053</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10764,16 +10981,16 @@
         <v>167</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>1058</v>
+        <v>1062</v>
       </c>
       <c r="D176" s="6" t="s">
-        <v>1059</v>
+        <v>1063</v>
       </c>
       <c r="E176" s="5" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10781,16 +10998,16 @@
         <v>168</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>1061</v>
+        <v>1065</v>
       </c>
       <c r="D177" s="6" t="s">
-        <v>1062</v>
+        <v>1066</v>
       </c>
       <c r="E177" s="5" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10798,16 +11015,16 @@
         <v>169</v>
       </c>
       <c r="B178" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="D178" s="6" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E178" s="5" t="s">
         <v>1064</v>
-      </c>
-      <c r="E178" s="5" t="s">
-        <v>1060</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10815,16 +11032,16 @@
         <v>170</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="D179" s="6" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="E179" s="5" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10832,16 +11049,16 @@
         <v>171</v>
       </c>
       <c r="B180" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="D180" s="6" t="s">
-        <v>1068</v>
+        <v>1072</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10849,16 +11066,16 @@
         <v>172</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
       <c r="D181" s="6" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10866,16 +11083,16 @@
         <v>173</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="D182" s="6" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="E182" s="5" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10883,16 +11100,16 @@
         <v>174</v>
       </c>
       <c r="B183" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>1075</v>
+        <v>1079</v>
       </c>
       <c r="D183" s="6" t="s">
-        <v>1076</v>
+        <v>1080</v>
       </c>
       <c r="E183" s="5" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10900,16 +11117,16 @@
         <v>175</v>
       </c>
       <c r="B184" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C184" s="5" t="s">
-        <v>1077</v>
+        <v>1081</v>
       </c>
       <c r="D184" s="6" t="s">
+        <v>1082</v>
+      </c>
+      <c r="E184" s="5" t="s">
         <v>1078</v>
-      </c>
-      <c r="E184" s="5" t="s">
-        <v>1074</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10917,16 +11134,16 @@
         <v>176</v>
       </c>
       <c r="B185" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C185" s="5" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="D185" s="6" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="E185" s="5" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10934,16 +11151,16 @@
         <v>177</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>1081</v>
+        <v>1085</v>
       </c>
       <c r="D186" s="6" t="s">
-        <v>1082</v>
+        <v>1086</v>
       </c>
       <c r="E186" s="5" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10951,16 +11168,16 @@
         <v>178</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C187" s="5" t="s">
-        <v>1083</v>
+        <v>1087</v>
       </c>
       <c r="D187" s="6" t="s">
-        <v>1084</v>
+        <v>1088</v>
       </c>
       <c r="E187" s="5" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10968,16 +11185,16 @@
         <v>179</v>
       </c>
       <c r="B188" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C188" s="5" t="s">
-        <v>1085</v>
+        <v>1089</v>
       </c>
       <c r="D188" s="6" t="s">
-        <v>1086</v>
+        <v>1090</v>
       </c>
       <c r="E188" s="5" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10985,16 +11202,16 @@
         <v>180</v>
       </c>
       <c r="B189" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C189" s="5" t="s">
-        <v>1088</v>
+        <v>1092</v>
       </c>
       <c r="D189" s="6" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="E189" s="5" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11002,16 +11219,16 @@
         <v>181</v>
       </c>
       <c r="B190" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="D190" s="6" t="s">
+        <v>1095</v>
+      </c>
+      <c r="E190" s="5" t="s">
         <v>1091</v>
-      </c>
-      <c r="E190" s="5" t="s">
-        <v>1087</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11019,16 +11236,16 @@
         <v>182</v>
       </c>
       <c r="B191" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C191" s="5" t="s">
-        <v>1092</v>
+        <v>1096</v>
       </c>
       <c r="D191" s="6" t="s">
-        <v>1093</v>
+        <v>1097</v>
       </c>
       <c r="E191" s="5" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11036,16 +11253,16 @@
         <v>183</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C192" s="5" t="s">
-        <v>1094</v>
+        <v>1098</v>
       </c>
       <c r="D192" s="6" t="s">
-        <v>1095</v>
+        <v>1099</v>
       </c>
       <c r="E192" s="5" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11053,13 +11270,13 @@
         <v>184</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C193" s="5" t="s">
-        <v>1096</v>
+        <v>1100</v>
       </c>
       <c r="D193" s="6" t="s">
-        <v>1097</v>
+        <v>1101</v>
       </c>
       <c r="E193" s="5" t="s">
         <v>533</v>
@@ -11070,16 +11287,16 @@
         <v>185</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>1098</v>
+        <v>1102</v>
       </c>
       <c r="D194" s="6" t="s">
-        <v>1099</v>
+        <v>1103</v>
       </c>
       <c r="E194" s="5" t="s">
-        <v>1100</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11087,16 +11304,16 @@
         <v>186</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C195" s="5" t="s">
-        <v>1101</v>
+        <v>1105</v>
       </c>
       <c r="D195" s="6" t="s">
-        <v>1102</v>
+        <v>1106</v>
       </c>
       <c r="E195" s="5" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11104,16 +11321,16 @@
         <v>187</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>1104</v>
+        <v>1108</v>
       </c>
       <c r="D196" s="6" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="E196" s="5" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11121,16 +11338,16 @@
         <v>188</v>
       </c>
       <c r="B197" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C197" s="5" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="D197" s="6" t="s">
+        <v>1111</v>
+      </c>
+      <c r="E197" s="5" t="s">
         <v>1107</v>
-      </c>
-      <c r="E197" s="5" t="s">
-        <v>1103</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11138,16 +11355,16 @@
         <v>189</v>
       </c>
       <c r="B198" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C198" s="5" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="D198" s="6" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="E198" s="5" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11155,16 +11372,16 @@
         <v>190</v>
       </c>
       <c r="B199" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C199" s="5" t="s">
-        <v>1110</v>
+        <v>1114</v>
       </c>
       <c r="D199" s="6" t="s">
-        <v>1111</v>
+        <v>1115</v>
       </c>
       <c r="E199" s="5" t="s">
-        <v>1112</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11172,16 +11389,16 @@
         <v>191</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C200" s="5" t="s">
-        <v>1113</v>
+        <v>1117</v>
       </c>
       <c r="D200" s="6" t="s">
-        <v>1114</v>
+        <v>1118</v>
       </c>
       <c r="E200" s="5" t="s">
-        <v>1112</v>
+        <v>1116</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11189,16 +11406,16 @@
         <v>192</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>1115</v>
+        <v>1119</v>
       </c>
       <c r="D201" s="6" t="s">
+        <v>1120</v>
+      </c>
+      <c r="E201" s="5" t="s">
         <v>1116</v>
-      </c>
-      <c r="E201" s="5" t="s">
-        <v>1112</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11206,16 +11423,16 @@
         <v>193</v>
       </c>
       <c r="B202" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C202" s="5" t="s">
-        <v>1117</v>
+        <v>1121</v>
       </c>
       <c r="D202" s="6" t="s">
-        <v>1118</v>
+        <v>1122</v>
       </c>
       <c r="E202" s="5" t="s">
-        <v>1119</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11223,16 +11440,16 @@
         <v>194</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>1120</v>
+        <v>1124</v>
       </c>
       <c r="D203" s="6" t="s">
-        <v>1121</v>
+        <v>1125</v>
       </c>
       <c r="E203" s="5" t="s">
-        <v>1119</v>
+        <v>1123</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11240,16 +11457,16 @@
         <v>195</v>
       </c>
       <c r="B204" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C204" s="5" t="s">
-        <v>1122</v>
+        <v>1126</v>
       </c>
       <c r="D204" s="6" t="s">
-        <v>1123</v>
+        <v>1127</v>
       </c>
       <c r="E204" s="5" t="s">
-        <v>1124</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11257,13 +11474,13 @@
         <v>196</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C205" s="5" t="s">
-        <v>1125</v>
+        <v>1129</v>
       </c>
       <c r="D205" s="6" t="s">
-        <v>1126</v>
+        <v>1130</v>
       </c>
       <c r="E205" s="5" t="s">
         <v>540</v>
@@ -11274,16 +11491,16 @@
         <v>197</v>
       </c>
       <c r="B206" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C206" s="5" t="s">
-        <v>1127</v>
+        <v>1131</v>
       </c>
       <c r="D206" s="6" t="s">
-        <v>1128</v>
+        <v>1132</v>
       </c>
       <c r="E206" s="5" t="s">
-        <v>1129</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11291,16 +11508,16 @@
         <v>198</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C207" s="5" t="s">
-        <v>1130</v>
+        <v>1134</v>
       </c>
       <c r="D207" s="6" t="s">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="E207" s="5" t="s">
-        <v>1129</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11308,16 +11525,16 @@
         <v>199</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C208" s="5" t="s">
-        <v>1132</v>
+        <v>1136</v>
       </c>
       <c r="D208" s="6" t="s">
+        <v>1137</v>
+      </c>
+      <c r="E208" s="5" t="s">
         <v>1133</v>
-      </c>
-      <c r="E208" s="5" t="s">
-        <v>1129</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11325,16 +11542,16 @@
         <v>200</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C209" s="5" t="s">
-        <v>1134</v>
+        <v>1138</v>
       </c>
       <c r="D209" s="6" t="s">
-        <v>1135</v>
+        <v>1139</v>
       </c>
       <c r="E209" s="5" t="s">
-        <v>1129</v>
+        <v>1133</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11342,16 +11559,16 @@
         <v>201</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C210" s="5" t="s">
-        <v>1136</v>
+        <v>1140</v>
       </c>
       <c r="D210" s="6" t="s">
-        <v>1137</v>
+        <v>1141</v>
       </c>
       <c r="E210" s="5" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11359,16 +11576,16 @@
         <v>202</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C211" s="5" t="s">
-        <v>1139</v>
+        <v>1143</v>
       </c>
       <c r="D211" s="6" t="s">
-        <v>1140</v>
+        <v>1144</v>
       </c>
       <c r="E211" s="5" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11376,152 +11593,305 @@
         <v>203</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C212" s="5" t="s">
-        <v>1141</v>
+        <v>1145</v>
       </c>
       <c r="D212" s="6" t="s">
+        <v>1146</v>
+      </c>
+      <c r="E212" s="5" t="s">
         <v>1142</v>
       </c>
-      <c r="E212" s="5" t="s">
-        <v>1138</v>
-      </c>
-    </row>
-    <row r="213" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="213" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="5" t="n">
         <v>204</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>1143</v>
+        <v>1147</v>
       </c>
       <c r="D213" s="6" t="s">
-        <v>1144</v>
+        <v>1148</v>
       </c>
       <c r="E213" s="5" t="s">
-        <v>1038</v>
-      </c>
-    </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1042</v>
+      </c>
+    </row>
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="5" t="n">
         <v>205</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C214" s="5" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="D214" s="6" t="s">
-        <v>1146</v>
+        <v>1150</v>
       </c>
       <c r="E214" s="5" t="s">
-        <v>1147</v>
-      </c>
-    </row>
-    <row r="215" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="215" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="5" t="n">
         <v>206</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C215" s="5" t="s">
-        <v>1148</v>
+        <v>1152</v>
       </c>
       <c r="D215" s="6" t="s">
-        <v>1149</v>
+        <v>1153</v>
       </c>
       <c r="E215" s="5" t="s">
-        <v>1150</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="5" t="n">
         <v>207</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C216" s="5" t="s">
-        <v>1151</v>
+        <v>1155</v>
       </c>
       <c r="D216" s="6" t="s">
-        <v>1152</v>
+        <v>1156</v>
       </c>
       <c r="E216" s="5" t="s">
-        <v>1150</v>
-      </c>
-    </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="5" t="n">
         <v>208</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="C217" s="5" t="s">
-        <v>1153</v>
+        <v>1157</v>
       </c>
       <c r="D217" s="6" t="s">
-        <v>1154</v>
+        <v>1158</v>
       </c>
       <c r="E217" s="5" t="s">
-        <v>1155</v>
-      </c>
-    </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="5" t="n">
         <v>209</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C218" s="5" t="s">
-        <v>1156</v>
+        <v>1160</v>
       </c>
       <c r="D218" s="6" t="s">
-        <v>1157</v>
+        <v>1161</v>
       </c>
       <c r="E218" s="5" t="s">
-        <v>1155</v>
-      </c>
-    </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="5" t="n">
         <v>210</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="C219" s="5" t="s">
-        <v>1158</v>
+        <v>1162</v>
       </c>
       <c r="D219" s="6" t="s">
+        <v>1163</v>
+      </c>
+      <c r="E219" s="5" t="s">
         <v>1159</v>
       </c>
-      <c r="E219" s="5" t="s">
-        <v>1155</v>
-      </c>
-    </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="5" t="n">
         <v>211</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="C220" s="5" t="s">
-        <v>1160</v>
+        <v>1164</v>
       </c>
       <c r="D220" s="6" t="s">
-        <v>1161</v>
+        <v>1165</v>
       </c>
       <c r="E220" s="5" t="s">
-        <v>1155</v>
+        <v>1159</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A221" s="5" t="n">
+        <v>212</v>
+      </c>
+      <c r="B221" s="5" t="s">
+        <v>860</v>
+      </c>
+      <c r="C221" s="5" t="s">
+        <v>1166</v>
+      </c>
+      <c r="D221" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E221" s="5" t="s">
+        <v>1168</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A222" s="5" t="n">
+        <v>213</v>
+      </c>
+      <c r="B222" s="5" t="s">
+        <v>665</v>
+      </c>
+      <c r="C222" s="5" t="s">
+        <v>1169</v>
+      </c>
+      <c r="D222" s="6" t="s">
+        <v>1170</v>
+      </c>
+      <c r="E222" s="5" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="5" t="n">
+        <v>214</v>
+      </c>
+      <c r="B223" s="5" t="s">
+        <v>860</v>
+      </c>
+      <c r="C223" s="5" t="s">
+        <v>1172</v>
+      </c>
+      <c r="D223" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="E223" s="5" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="5" t="n">
+        <v>215</v>
+      </c>
+      <c r="B224" s="5" t="s">
+        <v>860</v>
+      </c>
+      <c r="C224" s="5" t="s">
+        <v>1174</v>
+      </c>
+      <c r="D224" s="6" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E224" s="5" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="5" t="n">
+        <v>216</v>
+      </c>
+      <c r="B225" s="5" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C225" s="5" t="s">
+        <v>1176</v>
+      </c>
+      <c r="D225" s="6" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E225" s="5" t="s">
+        <v>1171</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="5" t="n">
+        <v>217</v>
+      </c>
+      <c r="B226" s="5" t="s">
+        <v>871</v>
+      </c>
+      <c r="C226" s="5" t="s">
+        <v>1178</v>
+      </c>
+      <c r="D226" s="6" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E226" s="5" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A227" s="5" t="n">
+        <v>218</v>
+      </c>
+      <c r="B227" s="5" t="s">
+        <v>665</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>1181</v>
+      </c>
+      <c r="D227" s="6" t="s">
+        <v>1182</v>
+      </c>
+      <c r="E227" s="5" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A228" s="5" t="n">
+        <v>219</v>
+      </c>
+      <c r="B228" s="5" t="s">
+        <v>804</v>
+      </c>
+      <c r="C228" s="5" t="s">
+        <v>1183</v>
+      </c>
+      <c r="D228" s="6" t="s">
+        <v>1184</v>
+      </c>
+      <c r="E228" s="5" t="s">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="229" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A229" s="5" t="n">
+        <v>220</v>
+      </c>
+      <c r="B229" s="5" t="s">
+        <v>1028</v>
+      </c>
+      <c r="C229" s="5" t="s">
+        <v>1185</v>
+      </c>
+      <c r="D229" s="6" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E229" s="5" t="s">
+        <v>1180</v>
       </c>
     </row>
   </sheetData>
@@ -11667,6 +12037,15 @@
     <hyperlink ref="D218" r:id="rId136" display="https://www.theguardian.com/commentisfree/2026/jul/17/trump-speech-election-denialism"/>
     <hyperlink ref="D219" r:id="rId137" display="https://www.cbsnews.com/news/trump-falsely-alleges-voting-machines-are-vulnerable-and-easily-compromised/"/>
     <hyperlink ref="D220" r:id="rId138" display="https://www.pbs.org/newshour/show/trump-tries-to-undermine-trust-in-elections-but-documents-dont-support-his-claims"/>
+    <hyperlink ref="D221" r:id="rId139" display="https://abcnews.com/Politics/wireStory/democratic-states-file-new-lawsuit-seeking-block-trumps-135974009"/>
+    <hyperlink ref="D222" r:id="rId140" display="https://www.nbcnews.com/politics/trump-administration/trump-orders-lake-ontario-renamed-lake-america-canada-trade-war-rcna594750"/>
+    <hyperlink ref="D223" r:id="rId141" display="https://abcnews.com/Politics/wireStory/group-democratic-senators-calls-ice-cancel-plan-buy-136008188"/>
+    <hyperlink ref="D224" r:id="rId142" display="https://abcnews.com/Politics/wireStory/us-goals-shifted-after-6-months-iran-war-135995683"/>
+    <hyperlink ref="D225" r:id="rId143" display="https://www.pbs.org/newshour/show/jan-6-rioters-pursue-new-path-for-payments-from-trump-administration"/>
+    <hyperlink ref="D226" r:id="rId144" display="https://www.npr.org/2026/08/28/nx-s1-5943238/trump-administration-proposal-would-allow-federal-grants-to-be-terminated-on-a-whim"/>
+    <hyperlink ref="D227" r:id="rId145" display="https://www.nbcnews.com/politics/trump-administration/trump-space-academy-nasa-military-rcna594870"/>
+    <hyperlink ref="D228" r:id="rId146" display="https://www.theguardian.com/politics/video/2026/aug/27/how-did-trump-get-so-rich-politics-weekly-america"/>
+    <hyperlink ref="D229" r:id="rId147" display="https://www.pbs.org/newshour/world/u-s-targets-egyptian-banks-uae-branches-under-new-push-for-irans-economic-isolation"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -11692,7 +12071,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>1162</v>
+        <v>1187</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -11701,7 +12080,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1163</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11710,7 +12089,7 @@
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A3)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11728,7 +12107,7 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A5)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11737,7 +12116,7 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A6)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11746,7 +12125,7 @@
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A7)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11773,7 +12152,7 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A10)</f>
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11791,7 +12170,7 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A12)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11859,11 +12238,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1164</v>
+        <v>1189</v>
       </c>
       <c r="B20" s="10" t="n">
         <f aca="false">SUM(B3:B19)</f>
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ingest approved entries (2026-09-06)
</commit_message>
<xml_diff>
--- a/data/Trump_Second_Term_Weekly_Tracker.xlsx
+++ b/data/Trump_Second_Term_Weekly_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$222</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Weekly Timeline'!$A$2:$F$226</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1778" uniqueCount="1190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1807" uniqueCount="1204">
   <si>
     <t xml:space="preserve">Documented actions and policies of the second Trump administration reported as harmful by major news outlets, courts, and government data — Jan 20, 2025 through Jul 8, 2026. One row per event; weeks with multiple events have multiple rows; quiet weeks are skipped. This compiles critical coverage as requested; the administration and its supporters dispute many of these characterizations. See the Sources tab (matching Ref #) and verify details independently before citing.</t>
   </si>
@@ -1680,6 +1680,18 @@
     <t xml:space="preserve">Aug 28</t>
   </si>
   <si>
+    <t xml:space="preserve">Aug 31, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infrastructure and History</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 4</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ref # matches the Source Ref column on the Weekly Timeline tab. URLs are provided where verified via current web results (mostly 2026 items). For 2025 items, outlet names and dates are given; searching the description text will locate the original coverage. Per your request the mix emphasizes CNN, Politico, MSNBC/MS NOW, NBC and independent outlets, alongside AP, Reuters, Guardian, NPR, CBS, ABC and court documents.</t>
   </si>
   <si>
@@ -3586,6 +3598,36 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.pbs.org/newshour/world/u-s-targets-egyptian-banks-uae-branches-under-new-push-for-irans-economic-isolation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOJ asks Supreme Court to allow Trump’s USPS action on mail-in ballots to proceed ahead of midterm elections</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/trump-administration/justice-department-usps-supreme-court-action-mail-ballots-elections-rcna595924</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 3, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavation work on Trump's arch in Washington to begin over next 2 weeks, administration says</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://abcnews.com/Politics/wireStory/excavation-work-trumps-arch-washington-begin-2-weeks-136185425</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trump administration rolls out 5 voter fraud prosecutions ahead of midterms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.nbcnews.com/politics/justice-department/trump-administration-rolls-5-voter-fraud-prosecutions-ahead-midterms-rcna596089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sep 4, 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Judge lets Pentagon move forward with firing Stars and Stripes journalists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.cbsnews.com/news/judge-allows-pentagon-fire-stars-stripes-journalists/</t>
   </si>
   <si>
     <t xml:space="preserve">Entries by category (live COUNTIF formulas against the Weekly Timeline tab)</t>
@@ -3774,7 +3816,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4067,7 +4109,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F222"/>
+  <dimension ref="A1:F226"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.01"/>
@@ -7997,7 +8039,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="5" t="s">
         <v>547</v>
       </c>
@@ -8013,7 +8055,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="5" t="s">
         <v>547</v>
       </c>
@@ -8029,7 +8071,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="5" t="s">
         <v>547</v>
       </c>
@@ -8045,7 +8087,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="5" t="s">
         <v>547</v>
       </c>
@@ -8061,7 +8103,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="5" t="s">
         <v>547</v>
       </c>
@@ -8077,7 +8119,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="5" t="s">
         <v>547</v>
       </c>
@@ -8093,7 +8135,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="5" t="s">
         <v>547</v>
       </c>
@@ -8109,7 +8151,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="5" t="s">
         <v>547</v>
       </c>
@@ -8125,7 +8167,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="5" t="s">
         <v>547</v>
       </c>
@@ -8139,8 +8181,72 @@
         <v>220</v>
       </c>
     </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A223" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B223" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="C223" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D223" s="4"/>
+      <c r="E223" s="4"/>
+      <c r="F223" s="4" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A224" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B224" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="C224" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="D224" s="4"/>
+      <c r="E224" s="4"/>
+      <c r="F224" s="4" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A225" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B225" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C225" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D225" s="4"/>
+      <c r="E225" s="4"/>
+      <c r="F225" s="4" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A226" s="4" t="s">
+        <v>551</v>
+      </c>
+      <c r="B226" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="C226" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D226" s="4"/>
+      <c r="E226" s="4"/>
+      <c r="F226" s="4" t="n">
+        <v>224</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:F222"/>
+  <autoFilter ref="A2:F226"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -8160,7 +8266,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E233"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
@@ -8171,7 +8277,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -8180,19 +8286,19 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8200,14 +8306,14 @@
         <v>1</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8215,14 +8321,14 @@
         <v>2</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8230,14 +8336,14 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8245,14 +8351,14 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8260,14 +8366,14 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8275,14 +8381,14 @@
         <v>6</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D8" s="5"/>
       <c r="E8" s="5" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8290,14 +8396,14 @@
         <v>7</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8305,14 +8411,14 @@
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8320,14 +8426,14 @@
         <v>9</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8335,14 +8441,14 @@
         <v>10</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8350,14 +8456,14 @@
         <v>11</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8365,14 +8471,14 @@
         <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8380,14 +8486,14 @@
         <v>13</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8395,14 +8501,14 @@
         <v>14</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8410,14 +8516,14 @@
         <v>15</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8425,14 +8531,14 @@
         <v>16</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8440,14 +8546,14 @@
         <v>17</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8455,14 +8561,14 @@
         <v>18</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8470,14 +8576,14 @@
         <v>19</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8485,14 +8591,14 @@
         <v>20</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8500,14 +8606,14 @@
         <v>21</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8515,14 +8621,14 @@
         <v>22</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8530,14 +8636,14 @@
         <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8545,14 +8651,14 @@
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8560,14 +8666,14 @@
         <v>25</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8575,14 +8681,14 @@
         <v>26</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8590,14 +8696,14 @@
         <v>27</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8605,14 +8711,14 @@
         <v>28</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8620,14 +8726,14 @@
         <v>29</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="D31" s="5"/>
       <c r="E31" s="5" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8635,14 +8741,14 @@
         <v>30</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D32" s="5"/>
       <c r="E32" s="5" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8650,14 +8756,14 @@
         <v>31</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="5" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8665,14 +8771,14 @@
         <v>32</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8680,14 +8786,14 @@
         <v>33</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="5" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8695,14 +8801,14 @@
         <v>34</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8710,14 +8816,14 @@
         <v>35</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8725,14 +8831,14 @@
         <v>36</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8740,14 +8846,14 @@
         <v>37</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8755,14 +8861,14 @@
         <v>38</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="D40" s="5"/>
       <c r="E40" s="5" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8770,10 +8876,10 @@
         <v>39</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="D41" s="5"/>
       <c r="E41" s="5" t="s">
@@ -8785,14 +8891,14 @@
         <v>40</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8800,14 +8906,14 @@
         <v>41</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="D43" s="5"/>
       <c r="E43" s="5" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8815,14 +8921,14 @@
         <v>42</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="D44" s="5"/>
       <c r="E44" s="5" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8830,14 +8936,14 @@
         <v>43</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8845,14 +8951,14 @@
         <v>44</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="D46" s="5"/>
       <c r="E46" s="5" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8860,14 +8966,14 @@
         <v>45</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="D47" s="5"/>
       <c r="E47" s="5" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8875,14 +8981,14 @@
         <v>46</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="D48" s="5"/>
       <c r="E48" s="5" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8890,14 +8996,14 @@
         <v>47</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8905,14 +9011,14 @@
         <v>48</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8920,14 +9026,14 @@
         <v>49</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="D51" s="5"/>
       <c r="E51" s="5" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8935,14 +9041,14 @@
         <v>50</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="D52" s="5"/>
       <c r="E52" s="5" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8950,14 +9056,14 @@
         <v>51</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="D53" s="5"/>
       <c r="E53" s="5" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8965,14 +9071,14 @@
         <v>52</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="D54" s="5"/>
       <c r="E54" s="5" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8980,14 +9086,14 @@
         <v>53</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="D55" s="5"/>
       <c r="E55" s="5" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8995,14 +9101,14 @@
         <v>54</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="D56" s="5"/>
       <c r="E56" s="5" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9010,14 +9116,14 @@
         <v>55</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="D57" s="5"/>
       <c r="E57" s="5" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9025,14 +9131,14 @@
         <v>56</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="D58" s="5"/>
       <c r="E58" s="5" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9040,14 +9146,14 @@
         <v>57</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="D59" s="5"/>
       <c r="E59" s="5" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9055,14 +9161,14 @@
         <v>58</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="D60" s="5"/>
       <c r="E60" s="5" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9070,14 +9176,14 @@
         <v>59</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="D61" s="5"/>
       <c r="E61" s="5" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9085,14 +9191,14 @@
         <v>60</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="D62" s="5"/>
       <c r="E62" s="5" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9100,14 +9206,14 @@
         <v>61</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="D63" s="5"/>
       <c r="E63" s="5" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9115,14 +9221,14 @@
         <v>62</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="D64" s="5"/>
       <c r="E64" s="5" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9130,14 +9236,14 @@
         <v>63</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="D65" s="5"/>
       <c r="E65" s="5" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9145,14 +9251,14 @@
         <v>64</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="D66" s="5"/>
       <c r="E66" s="5" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9160,14 +9266,14 @@
         <v>65</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="D67" s="5"/>
       <c r="E67" s="5" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9175,14 +9281,14 @@
         <v>66</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="D68" s="5"/>
       <c r="E68" s="5" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9190,14 +9296,14 @@
         <v>67</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="D69" s="5"/>
       <c r="E69" s="5" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9205,14 +9311,14 @@
         <v>68</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C70" s="5" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="D70" s="5"/>
       <c r="E70" s="5" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9220,14 +9326,14 @@
         <v>69</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C71" s="5" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="D71" s="5"/>
       <c r="E71" s="5" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9235,14 +9341,14 @@
         <v>70</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="D72" s="5"/>
       <c r="E72" s="5" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9250,14 +9356,14 @@
         <v>71</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="C73" s="5" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="D73" s="5"/>
       <c r="E73" s="5" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9265,14 +9371,14 @@
         <v>72</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="D74" s="5"/>
       <c r="E74" s="5" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9280,14 +9386,14 @@
         <v>73</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C75" s="5" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="D75" s="5"/>
       <c r="E75" s="5" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9295,14 +9401,14 @@
         <v>74</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="D76" s="5"/>
       <c r="E76" s="5" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9310,14 +9416,14 @@
         <v>75</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>770</v>
+        <v>774</v>
       </c>
       <c r="D77" s="5"/>
       <c r="E77" s="5" t="s">
-        <v>771</v>
+        <v>775</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9325,14 +9431,14 @@
         <v>76</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="D78" s="5"/>
       <c r="E78" s="5" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9340,14 +9446,14 @@
         <v>77</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>775</v>
+        <v>779</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="D79" s="5"/>
       <c r="E79" s="5" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9355,14 +9461,14 @@
         <v>78</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="D80" s="5"/>
       <c r="E80" s="5" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9370,14 +9476,14 @@
         <v>79</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="D81" s="5"/>
       <c r="E81" s="5" t="s">
-        <v>781</v>
+        <v>785</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9385,16 +9491,16 @@
         <v>80</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="C82" s="5" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9402,16 +9508,16 @@
         <v>81</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="C83" s="5" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9419,13 +9525,13 @@
         <v>82</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="C84" s="5" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>792</v>
+        <v>796</v>
       </c>
       <c r="E84" s="5" t="s">
         <v>297</v>
@@ -9436,13 +9542,13 @@
         <v>83</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>793</v>
+        <v>797</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>794</v>
+        <v>798</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="E85" s="5" t="s">
         <v>300</v>
@@ -9453,16 +9559,16 @@
         <v>84</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>798</v>
+        <v>802</v>
       </c>
       <c r="E86" s="5" t="s">
-        <v>799</v>
+        <v>803</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9470,16 +9576,16 @@
         <v>85</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>800</v>
+        <v>804</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>801</v>
+        <v>805</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>802</v>
+        <v>806</v>
       </c>
       <c r="E87" s="5" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9487,16 +9593,16 @@
         <v>86</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>805</v>
+        <v>809</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>806</v>
+        <v>810</v>
       </c>
       <c r="E88" s="5" t="s">
-        <v>803</v>
+        <v>807</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9504,16 +9610,16 @@
         <v>87</v>
       </c>
       <c r="B89" s="5" t="s">
+        <v>811</v>
+      </c>
+      <c r="C89" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>813</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>807</v>
-      </c>
-      <c r="C89" s="5" t="s">
-        <v>808</v>
-      </c>
-      <c r="D89" s="6" t="s">
-        <v>809</v>
-      </c>
-      <c r="E89" s="5" t="s">
-        <v>803</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9521,16 +9627,16 @@
         <v>88</v>
       </c>
       <c r="B90" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>811</v>
+        <v>815</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>812</v>
+        <v>816</v>
       </c>
       <c r="E90" s="5" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9538,16 +9644,16 @@
         <v>89</v>
       </c>
       <c r="B91" s="5" t="s">
-        <v>814</v>
+        <v>818</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>815</v>
+        <v>819</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>816</v>
+        <v>820</v>
       </c>
       <c r="E91" s="5" t="s">
-        <v>813</v>
+        <v>817</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9555,16 +9661,16 @@
         <v>90</v>
       </c>
       <c r="B92" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>817</v>
+        <v>821</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>818</v>
+        <v>822</v>
       </c>
       <c r="E92" s="5" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9572,16 +9678,16 @@
         <v>91</v>
       </c>
       <c r="B93" s="5" t="s">
-        <v>820</v>
+        <v>824</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>821</v>
+        <v>825</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>822</v>
+        <v>826</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9589,16 +9695,16 @@
         <v>92</v>
       </c>
       <c r="B94" s="5" t="s">
-        <v>823</v>
+        <v>827</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>824</v>
+        <v>828</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>825</v>
+        <v>829</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>826</v>
+        <v>830</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9606,16 +9712,16 @@
         <v>93</v>
       </c>
       <c r="B95" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>828</v>
+        <v>832</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9623,16 +9729,16 @@
         <v>94</v>
       </c>
       <c r="B96" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C96" s="5" t="s">
-        <v>830</v>
+        <v>834</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>831</v>
+        <v>835</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>829</v>
+        <v>833</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9640,16 +9746,16 @@
         <v>95</v>
       </c>
       <c r="B97" s="5" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="C97" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>838</v>
+      </c>
+      <c r="E97" s="5" t="s">
         <v>833</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>834</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>829</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9657,16 +9763,16 @@
         <v>96</v>
       </c>
       <c r="B98" s="5" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>835</v>
+        <v>839</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>836</v>
+        <v>840</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>819</v>
+        <v>823</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9674,16 +9780,16 @@
         <v>97</v>
       </c>
       <c r="B99" s="5" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C99" s="5" t="s">
-        <v>838</v>
+        <v>842</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>839</v>
+        <v>843</v>
       </c>
       <c r="E99" s="5" t="s">
-        <v>840</v>
+        <v>844</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9691,16 +9797,16 @@
         <v>98</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C100" s="5" t="s">
-        <v>841</v>
+        <v>845</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>842</v>
+        <v>846</v>
       </c>
       <c r="E100" s="5" t="s">
-        <v>843</v>
+        <v>847</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9708,16 +9814,16 @@
         <v>99</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>844</v>
+        <v>848</v>
       </c>
       <c r="D101" s="6" t="s">
-        <v>845</v>
+        <v>849</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>846</v>
+        <v>850</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9725,16 +9831,16 @@
         <v>100</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>847</v>
+        <v>851</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>848</v>
+        <v>852</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>849</v>
+        <v>853</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>850</v>
+        <v>854</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9742,16 +9848,16 @@
         <v>101</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>851</v>
+        <v>855</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>852</v>
+        <v>856</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9759,13 +9865,13 @@
         <v>102</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>352</v>
@@ -9776,16 +9882,16 @@
         <v>103</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="D105" s="6" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9793,16 +9899,16 @@
         <v>104</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="D106" s="6" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9810,16 +9916,16 @@
         <v>105</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9827,16 +9933,16 @@
         <v>106</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="D108" s="6" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9844,13 +9950,13 @@
         <v>107</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="D109" s="6" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>368</v>
@@ -9861,13 +9967,13 @@
         <v>108</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="D110" s="6" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>368</v>
@@ -9878,16 +9984,16 @@
         <v>109</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="D111" s="6" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9895,16 +10001,16 @@
         <v>110</v>
       </c>
       <c r="B112" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C112" s="5" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="D112" s="6" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9912,13 +10018,13 @@
         <v>111</v>
       </c>
       <c r="B113" s="5" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="C113" s="5" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="D113" s="6" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="E113" s="5" t="s">
         <v>382</v>
@@ -9929,16 +10035,16 @@
         <v>112</v>
       </c>
       <c r="B114" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C114" s="5" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="D114" s="6" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9946,16 +10052,16 @@
         <v>113</v>
       </c>
       <c r="B115" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C115" s="5" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="D115" s="6" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="E115" s="5" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9963,16 +10069,16 @@
         <v>114</v>
       </c>
       <c r="B116" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C116" s="5" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="D116" s="6" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="E116" s="5" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9980,16 +10086,16 @@
         <v>115</v>
       </c>
       <c r="B117" s="5" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="C117" s="5" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="D117" s="6" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="E117" s="5" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9997,13 +10103,13 @@
         <v>116</v>
       </c>
       <c r="B118" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C118" s="5" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="D118" s="6" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>396</v>
@@ -10014,16 +10120,16 @@
         <v>117</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="C119" s="5" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="D119" s="6" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="E119" s="5" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10031,16 +10137,16 @@
         <v>118</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C120" s="5" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="D120" s="6" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="E120" s="5" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10048,16 +10154,16 @@
         <v>119</v>
       </c>
       <c r="B121" s="5" t="s">
+        <v>910</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>911</v>
+      </c>
+      <c r="D121" s="6" t="s">
+        <v>912</v>
+      </c>
+      <c r="E121" s="5" t="s">
         <v>906</v>
-      </c>
-      <c r="C121" s="5" t="s">
-        <v>907</v>
-      </c>
-      <c r="D121" s="6" t="s">
-        <v>908</v>
-      </c>
-      <c r="E121" s="5" t="s">
-        <v>902</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10065,16 +10171,16 @@
         <v>120</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="C122" s="5" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="D122" s="6" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="E122" s="5" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10082,13 +10188,13 @@
         <v>121</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C123" s="5" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="E123" s="5" t="s">
         <v>409</v>
@@ -10099,13 +10205,13 @@
         <v>122</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C124" s="5" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="D124" s="6" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="E124" s="5" t="s">
         <v>409</v>
@@ -10116,16 +10222,16 @@
         <v>123</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C125" s="5" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="D125" s="6" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="E125" s="5" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
     </row>
     <row r="126" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10133,16 +10239,16 @@
         <v>124</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="C126" s="5" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="E126" s="5" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10150,16 +10256,16 @@
         <v>125</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="C127" s="5" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="D127" s="6" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="E127" s="5" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
     </row>
     <row r="128" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10167,16 +10273,16 @@
         <v>126</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="C128" s="5" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="D128" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E128" s="5" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10184,16 +10290,16 @@
         <v>127</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="C129" s="5" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="D129" s="6" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="E129" s="5" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10201,16 +10307,16 @@
         <v>128</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="C130" s="5" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="D130" s="6" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="E130" s="5" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10218,13 +10324,13 @@
         <v>129</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="C131" s="5" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
       <c r="D131" s="6" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="E131" s="5" t="s">
         <v>434</v>
@@ -10235,16 +10341,16 @@
         <v>130</v>
       </c>
       <c r="B132" s="5" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
       <c r="C132" s="5" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
       <c r="D132" s="6" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="E132" s="5" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10252,16 +10358,16 @@
         <v>131</v>
       </c>
       <c r="B133" s="5" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="C133" s="5" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="D133" s="6" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="E133" s="5" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10269,16 +10375,16 @@
         <v>132</v>
       </c>
       <c r="B134" s="5" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="C134" s="5" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="D134" s="6" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="E134" s="5" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10286,16 +10392,16 @@
         <v>133</v>
       </c>
       <c r="B135" s="5" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="C135" s="5" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="D135" s="6" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="E135" s="5" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10303,13 +10409,13 @@
         <v>134</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C136" s="5" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="D136" s="6" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>451</v>
@@ -10320,13 +10426,13 @@
         <v>135</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="C137" s="5" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="D137" s="6" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>451</v>
@@ -10337,16 +10443,16 @@
         <v>136</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>959</v>
+        <v>963</v>
       </c>
       <c r="C138" s="5" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="D138" s="6" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="E138" s="5" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10354,16 +10460,16 @@
         <v>137</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="C139" s="5" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="E139" s="5" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
     </row>
     <row r="140" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10371,13 +10477,13 @@
         <v>138</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>832</v>
+        <v>836</v>
       </c>
       <c r="C140" s="5" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>463</v>
@@ -10388,16 +10494,16 @@
         <v>139</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C141" s="5" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="D141" s="6" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="E141" s="5" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10405,16 +10511,16 @@
         <v>140</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="C142" s="5" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="E142" s="5" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10422,13 +10528,13 @@
         <v>141</v>
       </c>
       <c r="B143" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C143" s="5" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="D143" s="6" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>472</v>
@@ -10439,16 +10545,16 @@
         <v>142</v>
       </c>
       <c r="B144" s="5" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="C144" s="5" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="D144" s="6" t="s">
-        <v>980</v>
+        <v>984</v>
       </c>
       <c r="E144" s="5" t="s">
-        <v>981</v>
+        <v>985</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10456,13 +10562,13 @@
         <v>143</v>
       </c>
       <c r="B145" s="5" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C145" s="5" t="s">
-        <v>982</v>
+        <v>986</v>
       </c>
       <c r="D145" s="6" t="s">
-        <v>983</v>
+        <v>987</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>479</v>
@@ -10473,16 +10579,16 @@
         <v>144</v>
       </c>
       <c r="B146" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C146" s="5" t="s">
-        <v>984</v>
+        <v>988</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>985</v>
+        <v>989</v>
       </c>
       <c r="E146" s="5" t="s">
-        <v>986</v>
+        <v>990</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10490,16 +10596,16 @@
         <v>145</v>
       </c>
       <c r="B147" s="5" t="s">
-        <v>987</v>
+        <v>991</v>
       </c>
       <c r="C147" s="5" t="s">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="D147" s="6" t="s">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="E147" s="5" t="s">
-        <v>990</v>
+        <v>994</v>
       </c>
     </row>
     <row r="148" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10507,16 +10613,16 @@
         <v>146</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>991</v>
+        <v>995</v>
       </c>
       <c r="C148" s="5" t="s">
-        <v>992</v>
+        <v>996</v>
       </c>
       <c r="D148" s="6" t="s">
-        <v>993</v>
+        <v>997</v>
       </c>
       <c r="E148" s="5" t="s">
-        <v>994</v>
+        <v>998</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10524,13 +10630,13 @@
         <v>147</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>995</v>
+        <v>999</v>
       </c>
       <c r="C149" s="5" t="s">
-        <v>996</v>
+        <v>1000</v>
       </c>
       <c r="D149" s="6" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>492</v>
@@ -10541,13 +10647,13 @@
         <v>148</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>997</v>
+        <v>1001</v>
       </c>
       <c r="C150" s="5" t="s">
-        <v>998</v>
+        <v>1002</v>
       </c>
       <c r="D150" s="6" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>492</v>
@@ -10558,16 +10664,16 @@
         <v>149</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="C151" s="5" t="s">
-        <v>1000</v>
+        <v>1004</v>
       </c>
       <c r="D151" s="6" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="E151" s="5" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10575,16 +10681,16 @@
         <v>150</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>999</v>
+        <v>1003</v>
       </c>
       <c r="C152" s="5" t="s">
-        <v>1003</v>
+        <v>1007</v>
       </c>
       <c r="D152" s="6" t="s">
-        <v>1001</v>
+        <v>1005</v>
       </c>
       <c r="E152" s="5" t="s">
-        <v>1002</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="153" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10592,16 +10698,16 @@
         <v>151</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="C153" s="5" t="s">
-        <v>1005</v>
+        <v>1009</v>
       </c>
       <c r="D153" s="6" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10609,16 +10715,16 @@
         <v>152</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>1004</v>
+        <v>1008</v>
       </c>
       <c r="C154" s="5" t="s">
-        <v>1008</v>
+        <v>1012</v>
       </c>
       <c r="D154" s="6" t="s">
-        <v>1006</v>
+        <v>1010</v>
       </c>
       <c r="E154" s="5" t="s">
-        <v>1007</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="155" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10626,16 +10732,16 @@
         <v>153</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>1009</v>
+        <v>1013</v>
       </c>
       <c r="C155" s="5" t="s">
-        <v>1010</v>
+        <v>1014</v>
       </c>
       <c r="D155" s="6" t="s">
-        <v>1011</v>
+        <v>1015</v>
       </c>
       <c r="E155" s="5" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10643,16 +10749,16 @@
         <v>154</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>837</v>
+        <v>841</v>
       </c>
       <c r="C156" s="5" t="s">
-        <v>1013</v>
+        <v>1017</v>
       </c>
       <c r="D156" s="6" t="s">
-        <v>1014</v>
+        <v>1018</v>
       </c>
       <c r="E156" s="5" t="s">
-        <v>1012</v>
+        <v>1016</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10660,14 +10766,14 @@
         <v>155</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>1015</v>
+        <v>1019</v>
       </c>
       <c r="C157" s="5" t="s">
-        <v>1016</v>
+        <v>1020</v>
       </c>
       <c r="D157" s="5"/>
       <c r="E157" s="5" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="158" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10675,16 +10781,16 @@
         <v>156</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>1018</v>
+        <v>1022</v>
       </c>
       <c r="C158" s="5" t="s">
-        <v>1019</v>
+        <v>1023</v>
       </c>
       <c r="D158" s="6" t="s">
-        <v>1020</v>
+        <v>1024</v>
       </c>
       <c r="E158" s="5" t="s">
-        <v>1017</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10692,16 +10798,16 @@
         <v>157</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C159" s="5" t="s">
-        <v>1021</v>
+        <v>1025</v>
       </c>
       <c r="D159" s="6" t="s">
-        <v>1022</v>
+        <v>1026</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10709,16 +10815,16 @@
         <v>158</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C160" s="5" t="s">
-        <v>1024</v>
+        <v>1028</v>
       </c>
       <c r="D160" s="6" t="s">
-        <v>1025</v>
+        <v>1029</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10726,16 +10832,16 @@
         <v>159</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C161" s="5" t="s">
-        <v>1026</v>
+        <v>1030</v>
       </c>
       <c r="D161" s="6" t="s">
+        <v>1031</v>
+      </c>
+      <c r="E161" s="5" t="s">
         <v>1027</v>
-      </c>
-      <c r="E161" s="5" t="s">
-        <v>1023</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10743,16 +10849,16 @@
         <v>160</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C162" s="5" t="s">
-        <v>1029</v>
+        <v>1033</v>
       </c>
       <c r="D162" s="6" t="s">
-        <v>1030</v>
+        <v>1034</v>
       </c>
       <c r="E162" s="5" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10760,16 +10866,16 @@
         <v>161</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C163" s="5" t="s">
-        <v>1031</v>
+        <v>1035</v>
       </c>
       <c r="D163" s="6" t="s">
-        <v>1032</v>
+        <v>1036</v>
       </c>
       <c r="E163" s="5" t="s">
-        <v>1023</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10777,16 +10883,16 @@
         <v>162</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C164" s="5" t="s">
-        <v>1033</v>
+        <v>1037</v>
       </c>
       <c r="D164" s="6" t="s">
-        <v>1034</v>
+        <v>1038</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10794,16 +10900,16 @@
         <v>163</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C165" s="5" t="s">
-        <v>1036</v>
+        <v>1040</v>
       </c>
       <c r="D165" s="6" t="s">
-        <v>1037</v>
+        <v>1041</v>
       </c>
       <c r="E165" s="5" t="s">
-        <v>1035</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10811,13 +10917,13 @@
         <v>157</v>
       </c>
       <c r="B166" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C166" s="5" t="s">
-        <v>1038</v>
+        <v>1042</v>
       </c>
       <c r="D166" s="6" t="s">
-        <v>1039</v>
+        <v>1043</v>
       </c>
       <c r="E166" s="5" t="s">
         <v>521</v>
@@ -10828,16 +10934,16 @@
         <v>158</v>
       </c>
       <c r="B167" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C167" s="5" t="s">
-        <v>1040</v>
+        <v>1044</v>
       </c>
       <c r="D167" s="6" t="s">
-        <v>1041</v>
+        <v>1045</v>
       </c>
       <c r="E167" s="5" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="168" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10845,13 +10951,13 @@
         <v>159</v>
       </c>
       <c r="B168" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C168" s="5" t="s">
-        <v>1043</v>
+        <v>1047</v>
       </c>
       <c r="D168" s="6" t="s">
-        <v>1044</v>
+        <v>1048</v>
       </c>
       <c r="E168" s="5" t="s">
         <v>524</v>
@@ -10862,16 +10968,16 @@
         <v>160</v>
       </c>
       <c r="B169" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C169" s="5" t="s">
-        <v>1045</v>
+        <v>1049</v>
       </c>
       <c r="D169" s="6" t="s">
-        <v>1046</v>
+        <v>1050</v>
       </c>
       <c r="E169" s="5" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10879,16 +10985,16 @@
         <v>161</v>
       </c>
       <c r="B170" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C170" s="5" t="s">
-        <v>1048</v>
+        <v>1052</v>
       </c>
       <c r="D170" s="6" t="s">
-        <v>1049</v>
+        <v>1053</v>
       </c>
       <c r="E170" s="5" t="s">
-        <v>1047</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="171" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10896,16 +11002,16 @@
         <v>162</v>
       </c>
       <c r="B171" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C171" s="5" t="s">
-        <v>1050</v>
+        <v>1054</v>
       </c>
       <c r="D171" s="6" t="s">
+        <v>1055</v>
+      </c>
+      <c r="E171" s="5" t="s">
         <v>1051</v>
-      </c>
-      <c r="E171" s="5" t="s">
-        <v>1047</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10913,16 +11019,16 @@
         <v>163</v>
       </c>
       <c r="B172" s="5" t="s">
-        <v>810</v>
+        <v>814</v>
       </c>
       <c r="C172" s="5" t="s">
-        <v>1052</v>
+        <v>1056</v>
       </c>
       <c r="D172" s="6" t="s">
-        <v>1053</v>
+        <v>1057</v>
       </c>
       <c r="E172" s="5" t="s">
-        <v>1054</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10930,16 +11036,16 @@
         <v>164</v>
       </c>
       <c r="B173" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C173" s="5" t="s">
-        <v>1055</v>
+        <v>1059</v>
       </c>
       <c r="D173" s="6" t="s">
-        <v>1056</v>
+        <v>1060</v>
       </c>
       <c r="E173" s="5" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10947,16 +11053,16 @@
         <v>165</v>
       </c>
       <c r="B174" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C174" s="5" t="s">
-        <v>1058</v>
+        <v>1062</v>
       </c>
       <c r="D174" s="6" t="s">
-        <v>1059</v>
+        <v>1063</v>
       </c>
       <c r="E174" s="5" t="s">
-        <v>1057</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10964,16 +11070,16 @@
         <v>166</v>
       </c>
       <c r="B175" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C175" s="5" t="s">
-        <v>1060</v>
+        <v>1064</v>
       </c>
       <c r="D175" s="6" t="s">
+        <v>1065</v>
+      </c>
+      <c r="E175" s="5" t="s">
         <v>1061</v>
-      </c>
-      <c r="E175" s="5" t="s">
-        <v>1057</v>
       </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10981,16 +11087,16 @@
         <v>167</v>
       </c>
       <c r="B176" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C176" s="5" t="s">
-        <v>1062</v>
+        <v>1066</v>
       </c>
       <c r="D176" s="6" t="s">
-        <v>1063</v>
+        <v>1067</v>
       </c>
       <c r="E176" s="5" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10998,16 +11104,16 @@
         <v>168</v>
       </c>
       <c r="B177" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C177" s="5" t="s">
-        <v>1065</v>
+        <v>1069</v>
       </c>
       <c r="D177" s="6" t="s">
-        <v>1066</v>
+        <v>1070</v>
       </c>
       <c r="E177" s="5" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11015,16 +11121,16 @@
         <v>169</v>
       </c>
       <c r="B178" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>1067</v>
+        <v>1071</v>
       </c>
       <c r="D178" s="6" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E178" s="5" t="s">
         <v>1068</v>
-      </c>
-      <c r="E178" s="5" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11032,16 +11138,16 @@
         <v>170</v>
       </c>
       <c r="B179" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>1069</v>
+        <v>1073</v>
       </c>
       <c r="D179" s="6" t="s">
-        <v>1070</v>
+        <v>1074</v>
       </c>
       <c r="E179" s="5" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11049,16 +11155,16 @@
         <v>171</v>
       </c>
       <c r="B180" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>1071</v>
+        <v>1075</v>
       </c>
       <c r="D180" s="6" t="s">
-        <v>1072</v>
+        <v>1076</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>1064</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11066,16 +11172,16 @@
         <v>172</v>
       </c>
       <c r="B181" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>1073</v>
+        <v>1077</v>
       </c>
       <c r="D181" s="6" t="s">
-        <v>1074</v>
+        <v>1078</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>1075</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11083,16 +11189,16 @@
         <v>173</v>
       </c>
       <c r="B182" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>1076</v>
+        <v>1080</v>
       </c>
       <c r="D182" s="6" t="s">
-        <v>1077</v>
+        <v>1081</v>
       </c>
       <c r="E182" s="5" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="183" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11100,16 +11206,16 @@
         <v>174</v>
       </c>
       <c r="B183" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>1079</v>
+        <v>1083</v>
       </c>
       <c r="D183" s="6" t="s">
-        <v>1080</v>
+        <v>1084</v>
       </c>
       <c r="E183" s="5" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11117,16 +11223,16 @@
         <v>175</v>
       </c>
       <c r="B184" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C184" s="5" t="s">
-        <v>1081</v>
+        <v>1085</v>
       </c>
       <c r="D184" s="6" t="s">
+        <v>1086</v>
+      </c>
+      <c r="E184" s="5" t="s">
         <v>1082</v>
-      </c>
-      <c r="E184" s="5" t="s">
-        <v>1078</v>
       </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11134,16 +11240,16 @@
         <v>176</v>
       </c>
       <c r="B185" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C185" s="5" t="s">
-        <v>1083</v>
+        <v>1087</v>
       </c>
       <c r="D185" s="6" t="s">
-        <v>1084</v>
+        <v>1088</v>
       </c>
       <c r="E185" s="5" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11151,16 +11257,16 @@
         <v>177</v>
       </c>
       <c r="B186" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C186" s="5" t="s">
-        <v>1085</v>
+        <v>1089</v>
       </c>
       <c r="D186" s="6" t="s">
-        <v>1086</v>
+        <v>1090</v>
       </c>
       <c r="E186" s="5" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11168,16 +11274,16 @@
         <v>178</v>
       </c>
       <c r="B187" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C187" s="5" t="s">
-        <v>1087</v>
+        <v>1091</v>
       </c>
       <c r="D187" s="6" t="s">
-        <v>1088</v>
+        <v>1092</v>
       </c>
       <c r="E187" s="5" t="s">
-        <v>1078</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11185,16 +11291,16 @@
         <v>179</v>
       </c>
       <c r="B188" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C188" s="5" t="s">
-        <v>1089</v>
+        <v>1093</v>
       </c>
       <c r="D188" s="6" t="s">
-        <v>1090</v>
+        <v>1094</v>
       </c>
       <c r="E188" s="5" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11202,16 +11308,16 @@
         <v>180</v>
       </c>
       <c r="B189" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C189" s="5" t="s">
-        <v>1092</v>
+        <v>1096</v>
       </c>
       <c r="D189" s="6" t="s">
-        <v>1093</v>
+        <v>1097</v>
       </c>
       <c r="E189" s="5" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11219,16 +11325,16 @@
         <v>181</v>
       </c>
       <c r="B190" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C190" s="5" t="s">
-        <v>1094</v>
+        <v>1098</v>
       </c>
       <c r="D190" s="6" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E190" s="5" t="s">
         <v>1095</v>
-      </c>
-      <c r="E190" s="5" t="s">
-        <v>1091</v>
       </c>
     </row>
     <row r="191" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11236,16 +11342,16 @@
         <v>182</v>
       </c>
       <c r="B191" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C191" s="5" t="s">
-        <v>1096</v>
+        <v>1100</v>
       </c>
       <c r="D191" s="6" t="s">
-        <v>1097</v>
+        <v>1101</v>
       </c>
       <c r="E191" s="5" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11253,16 +11359,16 @@
         <v>183</v>
       </c>
       <c r="B192" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C192" s="5" t="s">
-        <v>1098</v>
+        <v>1102</v>
       </c>
       <c r="D192" s="6" t="s">
-        <v>1099</v>
+        <v>1103</v>
       </c>
       <c r="E192" s="5" t="s">
-        <v>1091</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11270,13 +11376,13 @@
         <v>184</v>
       </c>
       <c r="B193" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C193" s="5" t="s">
-        <v>1100</v>
+        <v>1104</v>
       </c>
       <c r="D193" s="6" t="s">
-        <v>1101</v>
+        <v>1105</v>
       </c>
       <c r="E193" s="5" t="s">
         <v>533</v>
@@ -11287,16 +11393,16 @@
         <v>185</v>
       </c>
       <c r="B194" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C194" s="5" t="s">
-        <v>1102</v>
+        <v>1106</v>
       </c>
       <c r="D194" s="6" t="s">
-        <v>1103</v>
+        <v>1107</v>
       </c>
       <c r="E194" s="5" t="s">
-        <v>1104</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11304,16 +11410,16 @@
         <v>186</v>
       </c>
       <c r="B195" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C195" s="5" t="s">
-        <v>1105</v>
+        <v>1109</v>
       </c>
       <c r="D195" s="6" t="s">
-        <v>1106</v>
+        <v>1110</v>
       </c>
       <c r="E195" s="5" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11321,16 +11427,16 @@
         <v>187</v>
       </c>
       <c r="B196" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>1108</v>
+        <v>1112</v>
       </c>
       <c r="D196" s="6" t="s">
-        <v>1109</v>
+        <v>1113</v>
       </c>
       <c r="E196" s="5" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11338,16 +11444,16 @@
         <v>188</v>
       </c>
       <c r="B197" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C197" s="5" t="s">
-        <v>1110</v>
+        <v>1114</v>
       </c>
       <c r="D197" s="6" t="s">
+        <v>1115</v>
+      </c>
+      <c r="E197" s="5" t="s">
         <v>1111</v>
-      </c>
-      <c r="E197" s="5" t="s">
-        <v>1107</v>
       </c>
     </row>
     <row r="198" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11355,16 +11461,16 @@
         <v>189</v>
       </c>
       <c r="B198" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C198" s="5" t="s">
-        <v>1112</v>
+        <v>1116</v>
       </c>
       <c r="D198" s="6" t="s">
-        <v>1113</v>
+        <v>1117</v>
       </c>
       <c r="E198" s="5" t="s">
-        <v>1107</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11372,16 +11478,16 @@
         <v>190</v>
       </c>
       <c r="B199" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C199" s="5" t="s">
-        <v>1114</v>
+        <v>1118</v>
       </c>
       <c r="D199" s="6" t="s">
-        <v>1115</v>
+        <v>1119</v>
       </c>
       <c r="E199" s="5" t="s">
-        <v>1116</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11389,16 +11495,16 @@
         <v>191</v>
       </c>
       <c r="B200" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C200" s="5" t="s">
-        <v>1117</v>
+        <v>1121</v>
       </c>
       <c r="D200" s="6" t="s">
-        <v>1118</v>
+        <v>1122</v>
       </c>
       <c r="E200" s="5" t="s">
-        <v>1116</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11406,16 +11512,16 @@
         <v>192</v>
       </c>
       <c r="B201" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>1119</v>
+        <v>1123</v>
       </c>
       <c r="D201" s="6" t="s">
+        <v>1124</v>
+      </c>
+      <c r="E201" s="5" t="s">
         <v>1120</v>
-      </c>
-      <c r="E201" s="5" t="s">
-        <v>1116</v>
       </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11423,16 +11529,16 @@
         <v>193</v>
       </c>
       <c r="B202" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C202" s="5" t="s">
-        <v>1121</v>
+        <v>1125</v>
       </c>
       <c r="D202" s="6" t="s">
-        <v>1122</v>
+        <v>1126</v>
       </c>
       <c r="E202" s="5" t="s">
-        <v>1123</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="203" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11440,16 +11546,16 @@
         <v>194</v>
       </c>
       <c r="B203" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>1124</v>
+        <v>1128</v>
       </c>
       <c r="D203" s="6" t="s">
-        <v>1125</v>
+        <v>1129</v>
       </c>
       <c r="E203" s="5" t="s">
-        <v>1123</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="204" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11457,16 +11563,16 @@
         <v>195</v>
       </c>
       <c r="B204" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C204" s="5" t="s">
-        <v>1126</v>
+        <v>1130</v>
       </c>
       <c r="D204" s="6" t="s">
-        <v>1127</v>
+        <v>1131</v>
       </c>
       <c r="E204" s="5" t="s">
-        <v>1128</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11474,13 +11580,13 @@
         <v>196</v>
       </c>
       <c r="B205" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C205" s="5" t="s">
-        <v>1129</v>
+        <v>1133</v>
       </c>
       <c r="D205" s="6" t="s">
-        <v>1130</v>
+        <v>1134</v>
       </c>
       <c r="E205" s="5" t="s">
         <v>540</v>
@@ -11491,16 +11597,16 @@
         <v>197</v>
       </c>
       <c r="B206" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C206" s="5" t="s">
-        <v>1131</v>
+        <v>1135</v>
       </c>
       <c r="D206" s="6" t="s">
-        <v>1132</v>
+        <v>1136</v>
       </c>
       <c r="E206" s="5" t="s">
-        <v>1133</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11508,16 +11614,16 @@
         <v>198</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C207" s="5" t="s">
-        <v>1134</v>
+        <v>1138</v>
       </c>
       <c r="D207" s="6" t="s">
-        <v>1135</v>
+        <v>1139</v>
       </c>
       <c r="E207" s="5" t="s">
-        <v>1133</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11525,16 +11631,16 @@
         <v>199</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C208" s="5" t="s">
-        <v>1136</v>
+        <v>1140</v>
       </c>
       <c r="D208" s="6" t="s">
+        <v>1141</v>
+      </c>
+      <c r="E208" s="5" t="s">
         <v>1137</v>
-      </c>
-      <c r="E208" s="5" t="s">
-        <v>1133</v>
       </c>
     </row>
     <row r="209" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11542,16 +11648,16 @@
         <v>200</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C209" s="5" t="s">
-        <v>1138</v>
+        <v>1142</v>
       </c>
       <c r="D209" s="6" t="s">
-        <v>1139</v>
+        <v>1143</v>
       </c>
       <c r="E209" s="5" t="s">
-        <v>1133</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="210" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11559,16 +11665,16 @@
         <v>201</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C210" s="5" t="s">
-        <v>1140</v>
+        <v>1144</v>
       </c>
       <c r="D210" s="6" t="s">
-        <v>1141</v>
+        <v>1145</v>
       </c>
       <c r="E210" s="5" t="s">
-        <v>1142</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11576,16 +11682,16 @@
         <v>202</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C211" s="5" t="s">
-        <v>1143</v>
+        <v>1147</v>
       </c>
       <c r="D211" s="6" t="s">
-        <v>1144</v>
+        <v>1148</v>
       </c>
       <c r="E211" s="5" t="s">
-        <v>1142</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="212" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11593,16 +11699,16 @@
         <v>203</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C212" s="5" t="s">
-        <v>1145</v>
+        <v>1149</v>
       </c>
       <c r="D212" s="6" t="s">
+        <v>1150</v>
+      </c>
+      <c r="E212" s="5" t="s">
         <v>1146</v>
-      </c>
-      <c r="E212" s="5" t="s">
-        <v>1142</v>
       </c>
     </row>
     <row r="213" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11610,16 +11716,16 @@
         <v>204</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>1147</v>
+        <v>1151</v>
       </c>
       <c r="D213" s="6" t="s">
-        <v>1148</v>
+        <v>1152</v>
       </c>
       <c r="E213" s="5" t="s">
-        <v>1042</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11627,16 +11733,16 @@
         <v>205</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C214" s="5" t="s">
-        <v>1149</v>
+        <v>1153</v>
       </c>
       <c r="D214" s="6" t="s">
-        <v>1150</v>
+        <v>1154</v>
       </c>
       <c r="E214" s="5" t="s">
-        <v>1151</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11644,16 +11750,16 @@
         <v>206</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C215" s="5" t="s">
-        <v>1152</v>
+        <v>1156</v>
       </c>
       <c r="D215" s="6" t="s">
-        <v>1153</v>
+        <v>1157</v>
       </c>
       <c r="E215" s="5" t="s">
-        <v>1154</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="216" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11661,16 +11767,16 @@
         <v>207</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C216" s="5" t="s">
-        <v>1155</v>
+        <v>1159</v>
       </c>
       <c r="D216" s="6" t="s">
-        <v>1156</v>
+        <v>1160</v>
       </c>
       <c r="E216" s="5" t="s">
-        <v>1154</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11678,16 +11784,16 @@
         <v>208</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C217" s="5" t="s">
-        <v>1157</v>
+        <v>1161</v>
       </c>
       <c r="D217" s="6" t="s">
-        <v>1158</v>
+        <v>1162</v>
       </c>
       <c r="E217" s="5" t="s">
-        <v>1159</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11695,16 +11801,16 @@
         <v>209</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C218" s="5" t="s">
-        <v>1160</v>
+        <v>1164</v>
       </c>
       <c r="D218" s="6" t="s">
-        <v>1161</v>
+        <v>1165</v>
       </c>
       <c r="E218" s="5" t="s">
-        <v>1159</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11712,16 +11818,16 @@
         <v>210</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C219" s="5" t="s">
-        <v>1162</v>
+        <v>1166</v>
       </c>
       <c r="D219" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E219" s="5" t="s">
         <v>1163</v>
-      </c>
-      <c r="E219" s="5" t="s">
-        <v>1159</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -11729,169 +11835,237 @@
         <v>211</v>
       </c>
       <c r="B220" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C220" s="5" t="s">
-        <v>1164</v>
+        <v>1168</v>
       </c>
       <c r="D220" s="6" t="s">
-        <v>1165</v>
+        <v>1169</v>
       </c>
       <c r="E220" s="5" t="s">
-        <v>1159</v>
-      </c>
-    </row>
-    <row r="221" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="221" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="5" t="n">
         <v>212</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C221" s="5" t="s">
-        <v>1166</v>
+        <v>1170</v>
       </c>
       <c r="D221" s="6" t="s">
-        <v>1167</v>
+        <v>1171</v>
       </c>
       <c r="E221" s="5" t="s">
-        <v>1168</v>
-      </c>
-    </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="5" t="n">
         <v>213</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C222" s="5" t="s">
-        <v>1169</v>
+        <v>1173</v>
       </c>
       <c r="D222" s="6" t="s">
-        <v>1170</v>
+        <v>1174</v>
       </c>
       <c r="E222" s="5" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="5" t="n">
         <v>214</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C223" s="5" t="s">
-        <v>1172</v>
+        <v>1176</v>
       </c>
       <c r="D223" s="6" t="s">
-        <v>1173</v>
+        <v>1177</v>
       </c>
       <c r="E223" s="5" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="224" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="224" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="5" t="n">
         <v>215</v>
       </c>
       <c r="B224" s="5" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="C224" s="5" t="s">
-        <v>1174</v>
+        <v>1178</v>
       </c>
       <c r="D224" s="6" t="s">
+        <v>1179</v>
+      </c>
+      <c r="E224" s="5" t="s">
         <v>1175</v>
       </c>
-      <c r="E224" s="5" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="5" t="n">
         <v>216</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C225" s="5" t="s">
-        <v>1176</v>
+        <v>1180</v>
       </c>
       <c r="D225" s="6" t="s">
-        <v>1177</v>
+        <v>1181</v>
       </c>
       <c r="E225" s="5" t="s">
-        <v>1171</v>
-      </c>
-    </row>
-    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="5" t="n">
         <v>217</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>1178</v>
+        <v>1182</v>
       </c>
       <c r="D226" s="6" t="s">
-        <v>1179</v>
+        <v>1183</v>
       </c>
       <c r="E226" s="5" t="s">
-        <v>1180</v>
-      </c>
-    </row>
-    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="5" t="n">
         <v>218</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="C227" s="5" t="s">
-        <v>1181</v>
+        <v>1185</v>
       </c>
       <c r="D227" s="6" t="s">
-        <v>1182</v>
+        <v>1186</v>
       </c>
       <c r="E227" s="5" t="s">
-        <v>1180</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="5" t="n">
         <v>219</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="C228" s="5" t="s">
-        <v>1183</v>
+        <v>1187</v>
       </c>
       <c r="D228" s="6" t="s">
+        <v>1188</v>
+      </c>
+      <c r="E228" s="5" t="s">
         <v>1184</v>
       </c>
-      <c r="E228" s="5" t="s">
-        <v>1180</v>
-      </c>
-    </row>
-    <row r="229" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="229" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="5" t="n">
         <v>220</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>1028</v>
+        <v>1032</v>
       </c>
       <c r="C229" s="5" t="s">
-        <v>1185</v>
+        <v>1189</v>
       </c>
       <c r="D229" s="6" t="s">
-        <v>1186</v>
+        <v>1190</v>
       </c>
       <c r="E229" s="5" t="s">
-        <v>1180</v>
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="230" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A230" s="5" t="n">
+        <v>221</v>
+      </c>
+      <c r="B230" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="C230" s="5" t="s">
+        <v>1191</v>
+      </c>
+      <c r="D230" s="6" t="s">
+        <v>1192</v>
+      </c>
+      <c r="E230" s="5" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A231" s="5" t="n">
+        <v>222</v>
+      </c>
+      <c r="B231" s="5" t="s">
+        <v>864</v>
+      </c>
+      <c r="C231" s="5" t="s">
+        <v>1194</v>
+      </c>
+      <c r="D231" s="6" t="s">
+        <v>1195</v>
+      </c>
+      <c r="E231" s="5" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A232" s="5" t="n">
+        <v>223</v>
+      </c>
+      <c r="B232" s="5" t="s">
+        <v>669</v>
+      </c>
+      <c r="C232" s="5" t="s">
+        <v>1196</v>
+      </c>
+      <c r="D232" s="6" t="s">
+        <v>1197</v>
+      </c>
+      <c r="E232" s="5" t="s">
+        <v>1198</v>
+      </c>
+    </row>
+    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A233" s="5" t="n">
+        <v>224</v>
+      </c>
+      <c r="B233" s="5" t="s">
+        <v>891</v>
+      </c>
+      <c r="C233" s="5" t="s">
+        <v>1199</v>
+      </c>
+      <c r="D233" s="6" t="s">
+        <v>1200</v>
+      </c>
+      <c r="E233" s="5" t="s">
+        <v>1198</v>
       </c>
     </row>
   </sheetData>
@@ -12046,6 +12220,10 @@
     <hyperlink ref="D227" r:id="rId145" display="https://www.nbcnews.com/politics/trump-administration/trump-space-academy-nasa-military-rcna594870"/>
     <hyperlink ref="D228" r:id="rId146" display="https://www.theguardian.com/politics/video/2026/aug/27/how-did-trump-get-so-rich-politics-weekly-america"/>
     <hyperlink ref="D229" r:id="rId147" display="https://www.pbs.org/newshour/world/u-s-targets-egyptian-banks-uae-branches-under-new-push-for-irans-economic-isolation"/>
+    <hyperlink ref="D230" r:id="rId148" display="https://www.nbcnews.com/politics/trump-administration/justice-department-usps-supreme-court-action-mail-ballots-elections-rcna595924"/>
+    <hyperlink ref="D231" r:id="rId149" display="https://abcnews.com/Politics/wireStory/excavation-work-trumps-arch-washington-begin-2-weeks-136185425"/>
+    <hyperlink ref="D232" r:id="rId150" display="https://www.nbcnews.com/politics/justice-department/trump-administration-rolls-5-voter-fraud-prosecutions-ahead-midterms-rcna596089"/>
+    <hyperlink ref="D233" r:id="rId151" display="https://www.cbsnews.com/news/judge-allows-pentagon-fire-stars-stripes-journalists/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -12062,7 +12240,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30.01"/>
@@ -12071,7 +12249,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="7" t="s">
-        <v>1187</v>
+        <v>1201</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -12080,7 +12258,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1188</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12116,7 +12294,7 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A6)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -12202,47 +12380,56 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>15</v>
+        <v>553</v>
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A16)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>68</v>
+        <v>15</v>
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A17)</f>
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A18)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>346</v>
+        <v>72</v>
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">COUNTIF('Weekly Timeline'!C:C,A19)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="B20" s="9" t="n">
+        <f aca="false">COUNTIF('Weekly Timeline'!C:C,A20)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
-        <v>1189</v>
-      </c>
-      <c r="B20" s="10" t="n">
-        <f aca="false">SUM(B3:B19)</f>
-        <v>164</v>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <f aca="false">SUM(B3:B20)</f>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>